<commit_message>
EH_Kurs: A3 certificates + original BG-Liste with 27 images
- Bescheinigungen: Paper size changed to A3 (landscape) for proper
  full-size certificate printing
- BG-Liste: Complete rebuild with original visual design:
  - All 27 PNG images embedded (green cross banner, borders,
    separators, stamp area) from original file
  - Original column widths (B=62.44, C=38.55, D=40.66)
  - Original row heights for all 43 rows per page
  - Original fonts (24pt company, 20pt names, 18pt fields)
  - Original green borders (#70D2A6) on participant cells
  - Conditional formatting to hide empty rows (white text)
  - 2 pages (10 participants each) with page break

https://claude.ai/code/session_0143BHkUCZBxvBT1DPHnv3wk
</commit_message>
<xml_diff>
--- a/EH_Kurs_2026.xlsx
+++ b/EH_Kurs_2026.xlsx
@@ -15,6 +15,7 @@
   </sheets>
   <definedNames>
     <definedName name="Lehrkraefte">Hilfslisten!$A$2:$A$20</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="2">'BG-Liste'!$A$1:$E$86</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -26,7 +27,7 @@
     <numFmt numFmtId="164" formatCode="DD.MM.YYYY"/>
     <numFmt numFmtId="165" formatCode="HH:MM"/>
   </numFmts>
-  <fonts count="21">
+  <fonts count="24">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -97,13 +98,29 @@
     </font>
     <font>
       <name val="Calibri"/>
-      <color rgb="00333333"/>
-      <sz val="10"/>
+      <color rgb="00000000"/>
+      <sz val="24"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="00000000"/>
+      <sz val="20"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="00000000"/>
+      <sz val="18"/>
     </font>
     <font>
       <name val="Calibri"/>
       <color rgb="00000000"/>
       <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00000000"/>
+      <sz val="14"/>
     </font>
     <font>
       <name val="Arial"/>
@@ -235,9 +252,6 @@
       </bottom>
     </border>
     <border>
-      <left style="medium">
-        <color rgb="0070D2A6"/>
-      </left>
       <right style="medium">
         <color rgb="0070D2A6"/>
       </right>
@@ -252,7 +266,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="53">
+  <cellXfs count="55">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -338,73 +352,75 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
+      <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="49" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="5" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="6" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="6" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="49" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="18" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="21" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -414,7 +430,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="1">
+  <dxfs count="2">
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -422,6 +438,11 @@
           <bgColor rgb="00FFCDD2"/>
         </patternFill>
       </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="00FFFFFF"/>
+      </font>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
@@ -494,6 +515,1361 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>0</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="11374437" cy="2048161"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>0</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="514422" cy="4277322"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="2" name="Image 2" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId2"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>4</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5601481" cy="314369"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="3" name="Image 3" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId3"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>2</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1810003" cy="2181529"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="4" name="Image 4" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId4"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>5</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5401429" cy="238157"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="5" name="Image 5" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId5"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>2</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="438211" cy="2486372"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="6" name="Image 6" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId6"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>2</col>
+      <colOff>0</colOff>
+      <row>5</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5544324" cy="304843"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="7" name="Image 7" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId7"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>2</col>
+      <colOff>0</colOff>
+      <row>3</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5410955" cy="476315"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="8" name="Image 8" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId8"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>6</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="11336332" cy="1086002"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="9" name="Image 9" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId9"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>7</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="533474" cy="6049219"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="10" name="Image 10" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId10"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>3</col>
+      <colOff>0</colOff>
+      <row>8</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1409897" cy="5296639"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="11" name="Image 11" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId11"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>19</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="11355385" cy="771633"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="12" name="Image 12" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId12"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>20</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1381318" cy="2734057"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="13" name="Image 13" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId13"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>23</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="6763694" cy="666843"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="14" name="Image 14" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId14"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>2</col>
+      <colOff>0</colOff>
+      <row>20</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="200053" cy="1943371"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="15" name="Image 15" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId15"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>2</col>
+      <colOff>0</colOff>
+      <row>24</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="790685" cy="314369"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="16" name="Image 16" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId16"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>3</col>
+      <colOff>0</colOff>
+      <row>24</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="3877216" cy="876422"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="17" name="Image 17" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId17"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>20</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="504895" cy="2162477"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="18" name="Image 18" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId18"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>25</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="11279174" cy="760400"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="19" name="Image 19" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId19"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>3</col>
+      <colOff>0</colOff>
+      <row>25</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1458493" cy="4727593"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="20" name="Image 20" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId20"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>31</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="10470280" cy="255763"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="21" name="Image 21" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId21"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>2</col>
+      <colOff>0</colOff>
+      <row>27</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="152421" cy="4242233"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="22" name="Image 22" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId22"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>29</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="10918018" cy="258657"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="23" name="Image 23" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId23"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>33</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="10813228" cy="275661"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="24" name="Image 24" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId24"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>39</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="10565543" cy="550839"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="25" name="Image 25" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId25"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>26</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="114316" cy="4196409"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="26" name="Image 26" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId26"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>39</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="724000" cy="266737"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="27" name="Image 27" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId27"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>43</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="11374437" cy="2048161"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="28" name="Image 28" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId28"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>43</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="514422" cy="4277322"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="29" name="Image 29" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId29"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>47</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5601481" cy="314369"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="30" name="Image 30" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId30"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>45</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1810003" cy="2181529"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="31" name="Image 31" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId31"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>48</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5401429" cy="238157"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="32" name="Image 32" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId32"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>45</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="438211" cy="2486372"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="33" name="Image 33" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId33"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>2</col>
+      <colOff>0</colOff>
+      <row>48</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5544324" cy="304843"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="34" name="Image 34" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId34"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>2</col>
+      <colOff>0</colOff>
+      <row>46</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5410955" cy="476315"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="35" name="Image 35" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId35"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>49</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="11336332" cy="1086002"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="36" name="Image 36" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId36"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>50</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="533474" cy="6049219"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="37" name="Image 37" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId37"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>3</col>
+      <colOff>0</colOff>
+      <row>51</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1409897" cy="5296639"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="38" name="Image 38" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId38"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>62</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="11355385" cy="771633"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="39" name="Image 39" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId39"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>63</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1381318" cy="2734057"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="40" name="Image 40" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId40"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>66</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="6763694" cy="666843"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="41" name="Image 41" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId41"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>2</col>
+      <colOff>0</colOff>
+      <row>63</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="200053" cy="1943371"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="42" name="Image 42" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId42"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>2</col>
+      <colOff>0</colOff>
+      <row>67</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="790685" cy="314369"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="43" name="Image 43" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId43"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>3</col>
+      <colOff>0</colOff>
+      <row>67</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="3877216" cy="876422"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="44" name="Image 44" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId44"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>63</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="504895" cy="2162477"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="45" name="Image 45" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId45"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>68</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="11279174" cy="760400"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="46" name="Image 46" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId46"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>3</col>
+      <colOff>0</colOff>
+      <row>68</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1458493" cy="4727593"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="47" name="Image 47" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId47"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>74</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="10470280" cy="255763"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="48" name="Image 48" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId48"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>2</col>
+      <colOff>0</colOff>
+      <row>70</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="152421" cy="4242233"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="49" name="Image 49" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId49"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>72</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="10918018" cy="258657"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="50" name="Image 50" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId50"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>76</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="10813228" cy="275661"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="51" name="Image 51" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId51"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>82</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="10565543" cy="550839"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="52" name="Image 52" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId52"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>69</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="114316" cy="4196409"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="53" name="Image 53" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId53"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>82</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="724000" cy="266737"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="54" name="Image 54" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId54"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -5579,7 +6955,7 @@
     <mergeCell ref="I155:O155"/>
   </mergeCells>
   <pageMargins left="0.4" right="0.4" top="0.4" bottom="0.4" header="0.3" footer="0.3"/>
-  <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
+  <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader>&amp;L&amp;1Internal</oddHeader>
     <oddFooter/>
@@ -5609,642 +6985,600 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E76"/>
+  <dimension ref="A5:D83"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="5" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="30" customWidth="1" min="5" max="5"/>
+    <col width="10.66" customWidth="1" min="1" max="1"/>
+    <col width="62.44" customWidth="1" min="2" max="2"/>
+    <col width="38.55" customWidth="1" min="3" max="3"/>
+    <col width="40.66" customWidth="1" min="4" max="4"/>
+    <col width="21.66" customWidth="1" min="5" max="5"/>
+    <col width="4.33" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
-    <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="29" t="inlineStr">
-        <is>
-          <t>Teilnehmerliste (BG)</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="6" customHeight="1"/>
-    <row r="3" ht="18" customHeight="1">
-      <c r="B3" s="30" t="inlineStr">
-        <is>
-          <t>Unternehmen:</t>
-        </is>
-      </c>
-      <c r="D3" s="30" t="inlineStr">
-        <is>
-          <t>BG / UV-Träger:</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="22" customHeight="1">
-      <c r="B4" s="31" t="inlineStr">
-        <is>
-          <t>Mercedes-Benz AG</t>
-        </is>
-      </c>
-      <c r="D4" s="31" t="inlineStr">
+    <row r="1" ht="42" customHeight="1"/>
+    <row r="2" ht="41.25" customHeight="1"/>
+    <row r="3" ht="38.25" customHeight="1"/>
+    <row r="4" ht="38.25" customHeight="1"/>
+    <row r="5" ht="42" customHeight="1">
+      <c r="B5" s="29" t="inlineStr">
+        <is>
+          <t>Mercedes Benz AG</t>
+        </is>
+      </c>
+      <c r="D5" s="30" t="inlineStr">
         <is>
           <t>BG-Metall Nord-Süd</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="22" customHeight="1">
-      <c r="B5" s="31" t="inlineStr">
-        <is>
-          <t>Mercedesstr. 1, 76437 Rastatt</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="6" customHeight="1"/>
-    <row r="7" ht="22" customHeight="1">
-      <c r="A7" s="7" t="inlineStr">
-        <is>
-          <t>Nr.</t>
-        </is>
-      </c>
-      <c r="B7" s="7" t="inlineStr">
-        <is>
-          <t>Nachname, Vorname</t>
-        </is>
-      </c>
-      <c r="D7" s="7" t="inlineStr">
-        <is>
-          <t>Geburtsdatum</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="26" customHeight="1">
-      <c r="A8" s="32" t="n">
+    <row r="6" ht="41.25" customHeight="1">
+      <c r="B6" s="31" t="inlineStr">
+        <is>
+          <t>Mercedesstr. 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="32.25" customHeight="1">
+      <c r="B7" s="31" t="inlineStr">
+        <is>
+          <t>76437 Rastatt</t>
+        </is>
+      </c>
+      <c r="D7" s="32" t="n"/>
+    </row>
+    <row r="8" ht="41.25" customHeight="1"/>
+    <row r="9" ht="34.5" customHeight="1"/>
+    <row r="10" ht="39.75" customHeight="1">
+      <c r="A10" s="33" t="n">
         <v>1</v>
       </c>
-      <c r="B8" s="33">
+      <c r="B10" s="34">
         <f>IF(Teilnehmer!B11&lt;&gt;"",Teilnehmer!B11&amp;", "&amp;Teilnehmer!C11,"")</f>
         <v/>
       </c>
-      <c r="D8" s="34">
+      <c r="C10" s="35">
         <f>IF(Teilnehmer!D11&lt;&gt;"",Teilnehmer!D11,"")</f>
         <v/>
       </c>
     </row>
-    <row r="9" ht="26" customHeight="1">
-      <c r="A9" s="35" t="n">
+    <row r="11" ht="39.75" customHeight="1">
+      <c r="A11" s="33" t="n">
         <v>2</v>
       </c>
-      <c r="B9" s="36">
+      <c r="B11" s="34">
         <f>IF(Teilnehmer!B12&lt;&gt;"",Teilnehmer!B12&amp;", "&amp;Teilnehmer!C12,"")</f>
         <v/>
       </c>
-      <c r="D9" s="37">
+      <c r="C11" s="35">
         <f>IF(Teilnehmer!D12&lt;&gt;"",Teilnehmer!D12,"")</f>
         <v/>
       </c>
     </row>
-    <row r="10" ht="26" customHeight="1">
-      <c r="A10" s="32" t="n">
+    <row r="12" ht="39.75" customHeight="1">
+      <c r="A12" s="33" t="n">
         <v>3</v>
       </c>
-      <c r="B10" s="33">
+      <c r="B12" s="34">
         <f>IF(Teilnehmer!B13&lt;&gt;"",Teilnehmer!B13&amp;", "&amp;Teilnehmer!C13,"")</f>
         <v/>
       </c>
-      <c r="D10" s="34">
+      <c r="C12" s="35">
         <f>IF(Teilnehmer!D13&lt;&gt;"",Teilnehmer!D13,"")</f>
         <v/>
       </c>
     </row>
-    <row r="11" ht="26" customHeight="1">
-      <c r="A11" s="35" t="n">
+    <row r="13" ht="39.75" customHeight="1">
+      <c r="A13" s="33" t="n">
         <v>4</v>
       </c>
-      <c r="B11" s="36">
+      <c r="B13" s="34">
         <f>IF(Teilnehmer!B14&lt;&gt;"",Teilnehmer!B14&amp;", "&amp;Teilnehmer!C14,"")</f>
         <v/>
       </c>
-      <c r="D11" s="37">
+      <c r="C13" s="35">
         <f>IF(Teilnehmer!D14&lt;&gt;"",Teilnehmer!D14,"")</f>
         <v/>
       </c>
     </row>
-    <row r="12" ht="26" customHeight="1">
-      <c r="A12" s="32" t="n">
+    <row r="14" ht="40.5" customHeight="1">
+      <c r="A14" s="33" t="n">
         <v>5</v>
       </c>
-      <c r="B12" s="33">
+      <c r="B14" s="34">
         <f>IF(Teilnehmer!B15&lt;&gt;"",Teilnehmer!B15&amp;", "&amp;Teilnehmer!C15,"")</f>
         <v/>
       </c>
-      <c r="D12" s="34">
+      <c r="C14" s="35">
         <f>IF(Teilnehmer!D15&lt;&gt;"",Teilnehmer!D15,"")</f>
         <v/>
       </c>
     </row>
-    <row r="13" ht="26" customHeight="1">
-      <c r="A13" s="35" t="n">
+    <row r="15" ht="39.75" customHeight="1">
+      <c r="A15" s="33" t="n">
         <v>6</v>
       </c>
-      <c r="B13" s="36">
+      <c r="B15" s="34">
         <f>IF(Teilnehmer!B16&lt;&gt;"",Teilnehmer!B16&amp;", "&amp;Teilnehmer!C16,"")</f>
         <v/>
       </c>
-      <c r="D13" s="37">
+      <c r="C15" s="35">
         <f>IF(Teilnehmer!D16&lt;&gt;"",Teilnehmer!D16,"")</f>
         <v/>
       </c>
     </row>
-    <row r="14" ht="26" customHeight="1">
-      <c r="A14" s="32" t="n">
+    <row r="16" ht="40.5" customHeight="1">
+      <c r="A16" s="33" t="n">
         <v>7</v>
       </c>
-      <c r="B14" s="33">
+      <c r="B16" s="34">
         <f>IF(Teilnehmer!B17&lt;&gt;"",Teilnehmer!B17&amp;", "&amp;Teilnehmer!C17,"")</f>
         <v/>
       </c>
-      <c r="D14" s="34">
+      <c r="C16" s="35">
         <f>IF(Teilnehmer!D17&lt;&gt;"",Teilnehmer!D17,"")</f>
         <v/>
       </c>
     </row>
-    <row r="15" ht="26" customHeight="1">
-      <c r="A15" s="35" t="n">
+    <row r="17" ht="39" customHeight="1">
+      <c r="A17" s="33" t="n">
         <v>8</v>
       </c>
-      <c r="B15" s="36">
+      <c r="B17" s="34">
         <f>IF(Teilnehmer!B18&lt;&gt;"",Teilnehmer!B18&amp;", "&amp;Teilnehmer!C18,"")</f>
         <v/>
       </c>
-      <c r="D15" s="37">
+      <c r="C17" s="35">
         <f>IF(Teilnehmer!D18&lt;&gt;"",Teilnehmer!D18,"")</f>
         <v/>
       </c>
     </row>
-    <row r="16" ht="26" customHeight="1">
-      <c r="A16" s="32" t="n">
+    <row r="18" ht="39.75" customHeight="1">
+      <c r="A18" s="33" t="n">
         <v>9</v>
       </c>
-      <c r="B16" s="33">
+      <c r="B18" s="34">
         <f>IF(Teilnehmer!B19&lt;&gt;"",Teilnehmer!B19&amp;", "&amp;Teilnehmer!C19,"")</f>
         <v/>
       </c>
-      <c r="D16" s="34">
+      <c r="C18" s="35">
         <f>IF(Teilnehmer!D19&lt;&gt;"",Teilnehmer!D19,"")</f>
         <v/>
       </c>
     </row>
-    <row r="17" ht="26" customHeight="1">
-      <c r="A17" s="35" t="n">
+    <row r="19" ht="39.75" customHeight="1">
+      <c r="A19" s="33" t="n">
         <v>10</v>
       </c>
-      <c r="B17" s="36">
+      <c r="B19" s="34">
         <f>IF(Teilnehmer!B20&lt;&gt;"",Teilnehmer!B20&amp;", "&amp;Teilnehmer!C20,"")</f>
         <v/>
       </c>
-      <c r="D17" s="37">
+      <c r="C19" s="35">
         <f>IF(Teilnehmer!D20&lt;&gt;"",Teilnehmer!D20,"")</f>
         <v/>
       </c>
     </row>
-    <row r="20">
-      <c r="B20" s="30" t="inlineStr">
-        <is>
-          <t>Ansprechpartner:</t>
-        </is>
-      </c>
-      <c r="C20" s="31" t="inlineStr">
+    <row r="20" ht="42" customHeight="1"/>
+    <row r="21" ht="27.75" customHeight="1"/>
+    <row r="22" ht="32.25" customHeight="1">
+      <c r="B22" s="36" t="inlineStr">
         <is>
           <t>Dr. Schmidt, Sabine</t>
         </is>
       </c>
-      <c r="D20" s="30" t="inlineStr">
-        <is>
-          <t>Lehrkraft:</t>
-        </is>
-      </c>
-      <c r="E20" s="31">
+    </row>
+    <row r="23" ht="32.25" customHeight="1">
+      <c r="B23" s="36" t="inlineStr">
+        <is>
+          <t>07222/91-22111</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="32.25" customHeight="1">
+      <c r="B24" s="37" t="inlineStr">
+        <is>
+          <t>sabine.m.schmidt@mercedes-benz.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="30" customHeight="1">
+      <c r="D25" s="38">
+        <f>Teilnehmer!C3</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26" ht="25.5" customHeight="1"/>
+    <row r="27" ht="31.5" customHeight="1"/>
+    <row r="28" ht="8.25" customHeight="1"/>
+    <row r="29" ht="25.5" customHeight="1">
+      <c r="C29" s="38">
+        <f>Teilnehmer!C3</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30" ht="16.5" customHeight="1"/>
+    <row r="31" ht="25.5" customHeight="1">
+      <c r="B31" s="39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  7.0103</t>
+        </is>
+      </c>
+      <c r="C31" s="40">
         <f>Teilnehmer!C4</f>
         <v/>
       </c>
     </row>
-    <row r="21">
-      <c r="B21" s="30" t="inlineStr">
-        <is>
-          <t>Telefon:</t>
-        </is>
-      </c>
-      <c r="C21" s="31" t="inlineStr">
+    <row r="32" ht="21" customHeight="1"/>
+    <row r="33" ht="26.25" customHeight="1">
+      <c r="B33" s="41">
+        <f>"  "&amp;Teilnehmer!C5</f>
+        <v/>
+      </c>
+      <c r="C33" s="40" t="inlineStr">
+        <is>
+          <t>Mercedes Benz AG, PKW Werk</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="15" customHeight="1"/>
+    <row r="35" ht="15" customHeight="1"/>
+    <row r="36" ht="29.25" customHeight="1">
+      <c r="C36" s="40" t="inlineStr">
+        <is>
+          <t>Mercedes Benz AG</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="29.25" customHeight="1">
+      <c r="C37" s="40" t="inlineStr">
+        <is>
+          <t>Werksärztlicher Dienst</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="29.25" customHeight="1">
+      <c r="C38" s="40" t="inlineStr">
+        <is>
+          <t>PKW-Werk Rastatt</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="29.25" customHeight="1">
+      <c r="C39" s="40" t="inlineStr">
+        <is>
+          <t>Mercedesstrasse 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="29.25" customHeight="1">
+      <c r="B40" s="38">
+        <f>Teilnehmer!C3</f>
+        <v/>
+      </c>
+      <c r="C40" s="40" t="inlineStr">
+        <is>
+          <t>76437 Rastatt</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="21" customHeight="1"/>
+    <row r="42" ht="9" customHeight="1"/>
+    <row r="43" ht="9" customHeight="1"/>
+    <row r="44" ht="42" customHeight="1"/>
+    <row r="45" ht="41.25" customHeight="1"/>
+    <row r="46" ht="38.25" customHeight="1"/>
+    <row r="47" ht="38.25" customHeight="1"/>
+    <row r="48" ht="42" customHeight="1">
+      <c r="B48" s="29" t="inlineStr">
+        <is>
+          <t>Mercedes Benz AG</t>
+        </is>
+      </c>
+      <c r="D48" s="30" t="inlineStr">
+        <is>
+          <t>BG-Metall Nord-Süd</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="41.25" customHeight="1">
+      <c r="B49" s="31" t="inlineStr">
+        <is>
+          <t>Mercedesstr. 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="32.25" customHeight="1">
+      <c r="B50" s="31" t="inlineStr">
+        <is>
+          <t>76437 Rastatt</t>
+        </is>
+      </c>
+      <c r="D50" s="32" t="n"/>
+    </row>
+    <row r="51" ht="41.25" customHeight="1"/>
+    <row r="52" ht="34.5" customHeight="1"/>
+    <row r="53" ht="39.75" customHeight="1">
+      <c r="A53" s="33" t="n">
+        <v>1</v>
+      </c>
+      <c r="B53" s="34">
+        <f>IF(Teilnehmer!B21&lt;&gt;"",Teilnehmer!B21&amp;", "&amp;Teilnehmer!C21,"")</f>
+        <v/>
+      </c>
+      <c r="C53" s="35">
+        <f>IF(Teilnehmer!D21&lt;&gt;"",Teilnehmer!D21,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="54" ht="39.75" customHeight="1">
+      <c r="A54" s="33" t="n">
+        <v>2</v>
+      </c>
+      <c r="B54" s="34">
+        <f>IF(Teilnehmer!B22&lt;&gt;"",Teilnehmer!B22&amp;", "&amp;Teilnehmer!C22,"")</f>
+        <v/>
+      </c>
+      <c r="C54" s="35">
+        <f>IF(Teilnehmer!D22&lt;&gt;"",Teilnehmer!D22,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="55" ht="39.75" customHeight="1">
+      <c r="A55" s="33" t="n">
+        <v>3</v>
+      </c>
+      <c r="B55" s="34">
+        <f>IF(Teilnehmer!B23&lt;&gt;"",Teilnehmer!B23&amp;", "&amp;Teilnehmer!C23,"")</f>
+        <v/>
+      </c>
+      <c r="C55" s="35">
+        <f>IF(Teilnehmer!D23&lt;&gt;"",Teilnehmer!D23,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="56" ht="39.75" customHeight="1">
+      <c r="A56" s="33" t="n">
+        <v>4</v>
+      </c>
+      <c r="B56" s="34">
+        <f>IF(Teilnehmer!B24&lt;&gt;"",Teilnehmer!B24&amp;", "&amp;Teilnehmer!C24,"")</f>
+        <v/>
+      </c>
+      <c r="C56" s="35">
+        <f>IF(Teilnehmer!D24&lt;&gt;"",Teilnehmer!D24,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="57" ht="40.5" customHeight="1">
+      <c r="A57" s="33" t="n">
+        <v>5</v>
+      </c>
+      <c r="B57" s="34">
+        <f>IF(Teilnehmer!B25&lt;&gt;"",Teilnehmer!B25&amp;", "&amp;Teilnehmer!C25,"")</f>
+        <v/>
+      </c>
+      <c r="C57" s="35">
+        <f>IF(Teilnehmer!D25&lt;&gt;"",Teilnehmer!D25,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="58" ht="39.75" customHeight="1">
+      <c r="A58" s="33" t="n">
+        <v>6</v>
+      </c>
+      <c r="B58" s="34">
+        <f>IF(Teilnehmer!B26&lt;&gt;"",Teilnehmer!B26&amp;", "&amp;Teilnehmer!C26,"")</f>
+        <v/>
+      </c>
+      <c r="C58" s="35">
+        <f>IF(Teilnehmer!D26&lt;&gt;"",Teilnehmer!D26,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="59" ht="40.5" customHeight="1">
+      <c r="A59" s="33" t="n">
+        <v>7</v>
+      </c>
+      <c r="B59" s="34">
+        <f>IF(Teilnehmer!B27&lt;&gt;"",Teilnehmer!B27&amp;", "&amp;Teilnehmer!C27,"")</f>
+        <v/>
+      </c>
+      <c r="C59" s="35">
+        <f>IF(Teilnehmer!D27&lt;&gt;"",Teilnehmer!D27,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="60" ht="39" customHeight="1">
+      <c r="A60" s="33" t="n">
+        <v>8</v>
+      </c>
+      <c r="B60" s="34">
+        <f>IF(Teilnehmer!B28&lt;&gt;"",Teilnehmer!B28&amp;", "&amp;Teilnehmer!C28,"")</f>
+        <v/>
+      </c>
+      <c r="C60" s="35">
+        <f>IF(Teilnehmer!D28&lt;&gt;"",Teilnehmer!D28,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="61" ht="39.75" customHeight="1">
+      <c r="A61" s="33" t="n">
+        <v>9</v>
+      </c>
+      <c r="B61" s="34">
+        <f>IF(Teilnehmer!B29&lt;&gt;"",Teilnehmer!B29&amp;", "&amp;Teilnehmer!C29,"")</f>
+        <v/>
+      </c>
+      <c r="C61" s="35">
+        <f>IF(Teilnehmer!D29&lt;&gt;"",Teilnehmer!D29,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="62" ht="39.75" customHeight="1">
+      <c r="A62" s="33" t="n">
+        <v>10</v>
+      </c>
+      <c r="B62" s="34">
+        <f>IF(Teilnehmer!B30&lt;&gt;"",Teilnehmer!B30&amp;", "&amp;Teilnehmer!C30,"")</f>
+        <v/>
+      </c>
+      <c r="C62" s="35">
+        <f>IF(Teilnehmer!D30&lt;&gt;"",Teilnehmer!D30,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="63" ht="42" customHeight="1"/>
+    <row r="64" ht="27.75" customHeight="1"/>
+    <row r="65" ht="32.25" customHeight="1">
+      <c r="B65" s="36" t="inlineStr">
+        <is>
+          <t>Dr. Schmidt, Sabine</t>
+        </is>
+      </c>
+    </row>
+    <row r="66" ht="32.25" customHeight="1">
+      <c r="B66" s="36" t="inlineStr">
         <is>
           <t>07222/91-22111</t>
         </is>
       </c>
-      <c r="D21" s="30" t="inlineStr">
-        <is>
-          <t>Datum:</t>
-        </is>
-      </c>
-      <c r="E21" s="38">
+    </row>
+    <row r="67" ht="32.25" customHeight="1">
+      <c r="B67" s="37" t="inlineStr">
+        <is>
+          <t>sabine.m.schmidt@mercedes-benz.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="68" ht="30" customHeight="1">
+      <c r="D68" s="38">
         <f>Teilnehmer!C3</f>
         <v/>
       </c>
     </row>
-    <row r="22">
-      <c r="B22" s="30" t="inlineStr">
-        <is>
-          <t>E-Mail:</t>
-        </is>
-      </c>
-      <c r="C22" s="31" t="inlineStr">
-        <is>
-          <t>sabine.m.schmidt@mercedes-benz.com</t>
-        </is>
-      </c>
-      <c r="D22" s="30" t="inlineStr">
-        <is>
-          <t>Registriernr.:</t>
-        </is>
-      </c>
-      <c r="E22" s="31">
-        <f>Teilnehmer!C5</f>
-        <v/>
-      </c>
-    </row>
-    <row r="23">
-      <c r="D23" s="30" t="inlineStr">
-        <is>
-          <t>QSEH-Kennziffer:</t>
-        </is>
-      </c>
-      <c r="E23" s="31" t="inlineStr">
-        <is>
-          <t>7.0103</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="B26" s="30" t="inlineStr">
-        <is>
-          <t>Stempel / Anschrift:</t>
-        </is>
-      </c>
-      <c r="D26" s="39" t="inlineStr">
-        <is>
-          <t>Mercedes-Benz AG, Werksärztlicher Dienst</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="D27" s="39" t="inlineStr">
-        <is>
-          <t>Mercedesstr. 1, 76437 Rastatt</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="B28" s="30" t="inlineStr">
-        <is>
-          <t>Datum:</t>
-        </is>
-      </c>
-      <c r="C28" s="38">
+    <row r="69" ht="25.5" customHeight="1"/>
+    <row r="70" ht="31.5" customHeight="1"/>
+    <row r="71" ht="8.25" customHeight="1"/>
+    <row r="72" ht="25.5" customHeight="1">
+      <c r="C72" s="38">
         <f>Teilnehmer!C3</f>
         <v/>
       </c>
     </row>
-    <row r="49" ht="28" customHeight="1">
-      <c r="A49" s="29" t="inlineStr">
-        <is>
-          <t>Teilnehmerliste (BG)</t>
-        </is>
-      </c>
-    </row>
-    <row r="50" ht="6" customHeight="1"/>
-    <row r="51" ht="18" customHeight="1">
-      <c r="B51" s="30" t="inlineStr">
-        <is>
-          <t>Unternehmen:</t>
-        </is>
-      </c>
-      <c r="D51" s="30" t="inlineStr">
-        <is>
-          <t>BG / UV-Träger:</t>
-        </is>
-      </c>
-    </row>
-    <row r="52" ht="22" customHeight="1">
-      <c r="B52" s="31" t="inlineStr">
-        <is>
-          <t>Mercedes-Benz AG</t>
-        </is>
-      </c>
-      <c r="D52" s="31" t="inlineStr">
-        <is>
-          <t>BG-Metall Nord-Süd</t>
-        </is>
-      </c>
-    </row>
-    <row r="53" ht="22" customHeight="1">
-      <c r="B53" s="31" t="inlineStr">
-        <is>
-          <t>Mercedesstr. 1, 76437 Rastatt</t>
-        </is>
-      </c>
-    </row>
-    <row r="54" ht="6" customHeight="1"/>
-    <row r="55" ht="22" customHeight="1">
-      <c r="A55" s="7" t="inlineStr">
-        <is>
-          <t>Nr.</t>
-        </is>
-      </c>
-      <c r="B55" s="7" t="inlineStr">
-        <is>
-          <t>Nachname, Vorname</t>
-        </is>
-      </c>
-      <c r="D55" s="7" t="inlineStr">
-        <is>
-          <t>Geburtsdatum</t>
-        </is>
-      </c>
-    </row>
-    <row r="56" ht="26" customHeight="1">
-      <c r="A56" s="32" t="n">
-        <v>1</v>
-      </c>
-      <c r="B56" s="33">
-        <f>IF(Teilnehmer!B21&lt;&gt;"",Teilnehmer!B21&amp;", "&amp;Teilnehmer!C21,"")</f>
-        <v/>
-      </c>
-      <c r="D56" s="34">
-        <f>IF(Teilnehmer!D21&lt;&gt;"",Teilnehmer!D21,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="57" ht="26" customHeight="1">
-      <c r="A57" s="35" t="n">
-        <v>2</v>
-      </c>
-      <c r="B57" s="36">
-        <f>IF(Teilnehmer!B22&lt;&gt;"",Teilnehmer!B22&amp;", "&amp;Teilnehmer!C22,"")</f>
-        <v/>
-      </c>
-      <c r="D57" s="37">
-        <f>IF(Teilnehmer!D22&lt;&gt;"",Teilnehmer!D22,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="58" ht="26" customHeight="1">
-      <c r="A58" s="32" t="n">
-        <v>3</v>
-      </c>
-      <c r="B58" s="33">
-        <f>IF(Teilnehmer!B23&lt;&gt;"",Teilnehmer!B23&amp;", "&amp;Teilnehmer!C23,"")</f>
-        <v/>
-      </c>
-      <c r="D58" s="34">
-        <f>IF(Teilnehmer!D23&lt;&gt;"",Teilnehmer!D23,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="59" ht="26" customHeight="1">
-      <c r="A59" s="35" t="n">
-        <v>4</v>
-      </c>
-      <c r="B59" s="36">
-        <f>IF(Teilnehmer!B24&lt;&gt;"",Teilnehmer!B24&amp;", "&amp;Teilnehmer!C24,"")</f>
-        <v/>
-      </c>
-      <c r="D59" s="37">
-        <f>IF(Teilnehmer!D24&lt;&gt;"",Teilnehmer!D24,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="60" ht="26" customHeight="1">
-      <c r="A60" s="32" t="n">
-        <v>5</v>
-      </c>
-      <c r="B60" s="33">
-        <f>IF(Teilnehmer!B25&lt;&gt;"",Teilnehmer!B25&amp;", "&amp;Teilnehmer!C25,"")</f>
-        <v/>
-      </c>
-      <c r="D60" s="34">
-        <f>IF(Teilnehmer!D25&lt;&gt;"",Teilnehmer!D25,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="61" ht="26" customHeight="1">
-      <c r="A61" s="35" t="n">
-        <v>6</v>
-      </c>
-      <c r="B61" s="36">
-        <f>IF(Teilnehmer!B26&lt;&gt;"",Teilnehmer!B26&amp;", "&amp;Teilnehmer!C26,"")</f>
-        <v/>
-      </c>
-      <c r="D61" s="37">
-        <f>IF(Teilnehmer!D26&lt;&gt;"",Teilnehmer!D26,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="62" ht="26" customHeight="1">
-      <c r="A62" s="32" t="n">
-        <v>7</v>
-      </c>
-      <c r="B62" s="33">
-        <f>IF(Teilnehmer!B27&lt;&gt;"",Teilnehmer!B27&amp;", "&amp;Teilnehmer!C27,"")</f>
-        <v/>
-      </c>
-      <c r="D62" s="34">
-        <f>IF(Teilnehmer!D27&lt;&gt;"",Teilnehmer!D27,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="63" ht="26" customHeight="1">
-      <c r="A63" s="35" t="n">
-        <v>8</v>
-      </c>
-      <c r="B63" s="36">
-        <f>IF(Teilnehmer!B28&lt;&gt;"",Teilnehmer!B28&amp;", "&amp;Teilnehmer!C28,"")</f>
-        <v/>
-      </c>
-      <c r="D63" s="37">
-        <f>IF(Teilnehmer!D28&lt;&gt;"",Teilnehmer!D28,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="64" ht="26" customHeight="1">
-      <c r="A64" s="32" t="n">
-        <v>9</v>
-      </c>
-      <c r="B64" s="33">
-        <f>IF(Teilnehmer!B29&lt;&gt;"",Teilnehmer!B29&amp;", "&amp;Teilnehmer!C29,"")</f>
-        <v/>
-      </c>
-      <c r="D64" s="34">
-        <f>IF(Teilnehmer!D29&lt;&gt;"",Teilnehmer!D29,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="65" ht="26" customHeight="1">
-      <c r="A65" s="35" t="n">
-        <v>10</v>
-      </c>
-      <c r="B65" s="36">
-        <f>IF(Teilnehmer!B30&lt;&gt;"",Teilnehmer!B30&amp;", "&amp;Teilnehmer!C30,"")</f>
-        <v/>
-      </c>
-      <c r="D65" s="37">
-        <f>IF(Teilnehmer!D30&lt;&gt;"",Teilnehmer!D30,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="68">
-      <c r="B68" s="30" t="inlineStr">
-        <is>
-          <t>Ansprechpartner:</t>
-        </is>
-      </c>
-      <c r="C68" s="31" t="inlineStr">
-        <is>
-          <t>Dr. Schmidt, Sabine</t>
-        </is>
-      </c>
-      <c r="D68" s="30" t="inlineStr">
-        <is>
-          <t>Lehrkraft:</t>
-        </is>
-      </c>
-      <c r="E68" s="31">
+    <row r="73" ht="16.5" customHeight="1"/>
+    <row r="74" ht="25.5" customHeight="1">
+      <c r="B74" s="39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  7.0103</t>
+        </is>
+      </c>
+      <c r="C74" s="40">
         <f>Teilnehmer!C4</f>
         <v/>
       </c>
     </row>
-    <row r="69">
-      <c r="B69" s="30" t="inlineStr">
-        <is>
-          <t>Telefon:</t>
-        </is>
-      </c>
-      <c r="C69" s="31" t="inlineStr">
-        <is>
-          <t>07222/91-22111</t>
-        </is>
-      </c>
-      <c r="D69" s="30" t="inlineStr">
-        <is>
-          <t>Datum:</t>
-        </is>
-      </c>
-      <c r="E69" s="38">
+    <row r="75" ht="21" customHeight="1"/>
+    <row r="76" ht="26.25" customHeight="1">
+      <c r="B76" s="41">
+        <f>"  "&amp;Teilnehmer!C5</f>
+        <v/>
+      </c>
+      <c r="C76" s="40" t="inlineStr">
+        <is>
+          <t>Mercedes Benz AG, PKW Werk</t>
+        </is>
+      </c>
+    </row>
+    <row r="77" ht="15" customHeight="1"/>
+    <row r="78" ht="15" customHeight="1"/>
+    <row r="79" ht="29.25" customHeight="1">
+      <c r="C79" s="40" t="inlineStr">
+        <is>
+          <t>Mercedes Benz AG</t>
+        </is>
+      </c>
+    </row>
+    <row r="80" ht="29.25" customHeight="1">
+      <c r="C80" s="40" t="inlineStr">
+        <is>
+          <t>Werksärztlicher Dienst</t>
+        </is>
+      </c>
+    </row>
+    <row r="81" ht="29.25" customHeight="1">
+      <c r="C81" s="40" t="inlineStr">
+        <is>
+          <t>PKW-Werk Rastatt</t>
+        </is>
+      </c>
+    </row>
+    <row r="82" ht="29.25" customHeight="1">
+      <c r="C82" s="40" t="inlineStr">
+        <is>
+          <t>Mercedesstrasse 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="83" ht="29.25" customHeight="1">
+      <c r="B83" s="38">
         <f>Teilnehmer!C3</f>
         <v/>
       </c>
-    </row>
-    <row r="70">
-      <c r="B70" s="30" t="inlineStr">
-        <is>
-          <t>E-Mail:</t>
-        </is>
-      </c>
-      <c r="C70" s="31" t="inlineStr">
-        <is>
-          <t>sabine.m.schmidt@mercedes-benz.com</t>
-        </is>
-      </c>
-      <c r="D70" s="30" t="inlineStr">
-        <is>
-          <t>Registriernr.:</t>
-        </is>
-      </c>
-      <c r="E70" s="31">
-        <f>Teilnehmer!C5</f>
-        <v/>
-      </c>
-    </row>
-    <row r="71">
-      <c r="D71" s="30" t="inlineStr">
-        <is>
-          <t>QSEH-Kennziffer:</t>
-        </is>
-      </c>
-      <c r="E71" s="31" t="inlineStr">
-        <is>
-          <t>7.0103</t>
-        </is>
-      </c>
-    </row>
-    <row r="74">
-      <c r="B74" s="30" t="inlineStr">
-        <is>
-          <t>Stempel / Anschrift:</t>
-        </is>
-      </c>
-      <c r="D74" s="39" t="inlineStr">
-        <is>
-          <t>Mercedes-Benz AG, Werksärztlicher Dienst</t>
-        </is>
-      </c>
-    </row>
-    <row r="75">
-      <c r="D75" s="39" t="inlineStr">
-        <is>
-          <t>Mercedesstr. 1, 76437 Rastatt</t>
-        </is>
-      </c>
-    </row>
-    <row r="76">
-      <c r="B76" s="30" t="inlineStr">
-        <is>
-          <t>Datum:</t>
-        </is>
-      </c>
-      <c r="C76" s="38">
-        <f>Teilnehmer!C3</f>
-        <v/>
-      </c>
-    </row>
+      <c r="C83" s="40" t="inlineStr">
+        <is>
+          <t>76437 Rastatt</t>
+        </is>
+      </c>
+    </row>
+    <row r="84" ht="21" customHeight="1"/>
+    <row r="85" ht="9" customHeight="1"/>
+    <row r="86" ht="9" customHeight="1"/>
   </sheetData>
-  <mergeCells count="34">
-    <mergeCell ref="B16:C16"/>
-    <mergeCell ref="B62:C62"/>
-    <mergeCell ref="B7:C7"/>
-    <mergeCell ref="B3:C3"/>
-    <mergeCell ref="B59:C59"/>
-    <mergeCell ref="B56:C56"/>
-    <mergeCell ref="B12:C12"/>
-    <mergeCell ref="B58:C58"/>
-    <mergeCell ref="B52:C52"/>
-    <mergeCell ref="B11:C11"/>
-    <mergeCell ref="D27:E27"/>
-    <mergeCell ref="B61:C61"/>
-    <mergeCell ref="B14:C14"/>
-    <mergeCell ref="B60:C60"/>
-    <mergeCell ref="B17:C17"/>
-    <mergeCell ref="B57:C57"/>
-    <mergeCell ref="B8:C8"/>
-    <mergeCell ref="B53:C53"/>
-    <mergeCell ref="D75:E75"/>
-    <mergeCell ref="B13:C13"/>
-    <mergeCell ref="B10:C10"/>
-    <mergeCell ref="B9:C9"/>
-    <mergeCell ref="B65:C65"/>
-    <mergeCell ref="B55:C55"/>
-    <mergeCell ref="D74:E74"/>
-    <mergeCell ref="A49:C49"/>
-    <mergeCell ref="B15:C15"/>
-    <mergeCell ref="B64:C64"/>
-    <mergeCell ref="A1:C1"/>
-    <mergeCell ref="B5:C5"/>
-    <mergeCell ref="B51:C51"/>
-    <mergeCell ref="B63:C63"/>
-    <mergeCell ref="D26:E26"/>
-    <mergeCell ref="B4:C4"/>
+  <mergeCells count="16">
+    <mergeCell ref="C83:D83"/>
+    <mergeCell ref="C29:D29"/>
+    <mergeCell ref="C38:D38"/>
+    <mergeCell ref="C80:D80"/>
+    <mergeCell ref="C72:D72"/>
+    <mergeCell ref="C82:D82"/>
+    <mergeCell ref="C33:D33"/>
+    <mergeCell ref="C81:D81"/>
+    <mergeCell ref="C76:D76"/>
+    <mergeCell ref="C37:D37"/>
+    <mergeCell ref="C36:D36"/>
+    <mergeCell ref="C74:D74"/>
+    <mergeCell ref="C40:D40"/>
+    <mergeCell ref="C31:D31"/>
+    <mergeCell ref="C79:D79"/>
+    <mergeCell ref="C39:D39"/>
   </mergeCells>
-  <pageMargins left="0.5" right="0.5" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
+  <conditionalFormatting sqref="B10:B19">
+    <cfRule type="cellIs" priority="1" operator="equal" dxfId="1">
+      <formula>", "</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C10:C19">
+    <cfRule type="cellIs" priority="2" operator="equal" dxfId="1">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B53:B62">
+    <cfRule type="cellIs" priority="3" operator="equal" dxfId="1">
+      <formula>", "</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C53:C62">
+    <cfRule type="cellIs" priority="4" operator="equal" dxfId="1">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.197" right="0.079" top="0.394" bottom="0.394" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" paperSize="9" fitToHeight="0" fitToWidth="1"/>
   <rowBreaks count="1" manualBreakCount="1">
-    <brk id="48" min="0" max="16383" man="1"/>
+    <brk id="43" min="0" max="16383" man="1"/>
   </rowBreaks>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -6268,221 +7602,221 @@
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
-      <c r="A1" s="40" t="inlineStr">
+      <c r="A1" s="42" t="inlineStr">
         <is>
           <t>Lehrgangsdokumentation</t>
         </is>
       </c>
     </row>
     <row r="2" ht="18" customHeight="1">
-      <c r="A2" s="41" t="inlineStr">
+      <c r="A2" s="43" t="inlineStr">
         <is>
           <t>gem. Abschnitt 2.4.6 DGUV Grundsatz 304-001</t>
         </is>
       </c>
     </row>
     <row r="4" ht="22" customHeight="1">
-      <c r="B4" s="42" t="inlineStr">
+      <c r="B4" s="44" t="inlineStr">
         <is>
           <t>Angaben zur Ausbildungsstelle</t>
         </is>
       </c>
     </row>
     <row r="5" ht="14" customHeight="1">
-      <c r="B5" s="43" t="inlineStr">
+      <c r="B5" s="45" t="inlineStr">
         <is>
           <t>Bezeichnung</t>
         </is>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1">
-      <c r="B6" s="44" t="inlineStr">
+      <c r="B6" s="46" t="inlineStr">
         <is>
           <t>Mercedes-Benz AG</t>
         </is>
       </c>
-      <c r="E6" s="45" t="inlineStr">
+      <c r="E6" s="47" t="inlineStr">
         <is>
           <t>QSEH-Kennziffer:</t>
         </is>
       </c>
-      <c r="F6" s="44">
+      <c r="F6" s="46">
         <f>Teilnehmer!F5</f>
         <v/>
       </c>
     </row>
     <row r="8" ht="14" customHeight="1">
-      <c r="B8" s="43" t="inlineStr">
+      <c r="B8" s="45" t="inlineStr">
         <is>
           <t>Straße / Hausnr.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="20" customHeight="1">
-      <c r="B9" s="44" t="inlineStr">
+      <c r="B9" s="46" t="inlineStr">
         <is>
           <t>Mercedesstr. 1</t>
         </is>
       </c>
     </row>
     <row r="11" ht="14" customHeight="1">
-      <c r="B11" s="43" t="inlineStr">
+      <c r="B11" s="45" t="inlineStr">
         <is>
           <t>PLZ / Ort</t>
         </is>
       </c>
     </row>
     <row r="12" ht="20" customHeight="1">
-      <c r="B12" s="44" t="inlineStr">
+      <c r="B12" s="46" t="inlineStr">
         <is>
           <t>76437 Rastatt</t>
         </is>
       </c>
     </row>
     <row r="14" ht="22" customHeight="1">
-      <c r="B14" s="42" t="inlineStr">
+      <c r="B14" s="44" t="inlineStr">
         <is>
           <t>Angaben zum Seminar</t>
         </is>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1">
-      <c r="B15" s="46">
+      <c r="B15" s="48">
         <f>IF(Teilnehmer!F4="EH-Ausbildung","X","  ")&amp;" EH-Ausbildung       "&amp;IF(Teilnehmer!F4="EH-Fortbildung","X","  ")&amp;" EH-Fortbildung       "&amp;IF(Teilnehmer!F4="EH-Schulung","X","  ")&amp;" EH-Schulung"</f>
         <v/>
       </c>
     </row>
     <row r="17" ht="20" customHeight="1">
-      <c r="B17" s="45" t="inlineStr">
+      <c r="B17" s="47" t="inlineStr">
         <is>
           <t>Registriernummer:</t>
         </is>
       </c>
-      <c r="C17" s="44">
+      <c r="C17" s="46">
         <f>Teilnehmer!C5</f>
         <v/>
       </c>
-      <c r="E17" s="45" t="inlineStr">
+      <c r="E17" s="47" t="inlineStr">
         <is>
           <t>Lehrgangsort:</t>
         </is>
       </c>
-      <c r="F17" s="44" t="inlineStr">
+      <c r="F17" s="46" t="inlineStr">
         <is>
           <t>Mercedes-Benz AG, PKW-Werk Rastatt</t>
         </is>
       </c>
     </row>
     <row r="18" ht="14" customHeight="1">
-      <c r="B18" s="43" t="inlineStr">
+      <c r="B18" s="45" t="inlineStr">
         <is>
           <t>(aus dem QSEH-Portal)</t>
         </is>
       </c>
-      <c r="F18" s="43" t="inlineStr">
+      <c r="F18" s="45" t="inlineStr">
         <is>
           <t>Gebäude 39, Gesundheitszentrum 1.OG</t>
         </is>
       </c>
     </row>
     <row r="20" ht="20" customHeight="1">
-      <c r="B20" s="45" t="inlineStr">
+      <c r="B20" s="47" t="inlineStr">
         <is>
           <t>Lehrgangsdatum:</t>
         </is>
       </c>
-      <c r="C20" s="47">
+      <c r="C20" s="49">
         <f>Teilnehmer!C3</f>
         <v/>
       </c>
-      <c r="E20" s="45" t="inlineStr">
+      <c r="E20" s="47" t="inlineStr">
         <is>
           <t>Uhrzeit:</t>
         </is>
       </c>
-      <c r="F20" s="44">
+      <c r="F20" s="46">
         <f>"von "&amp;TEXT(Teilnehmer!F3,"HH:MM")&amp;" Uhr bis "&amp;TEXT(Teilnehmer!H3,"HH:MM")&amp;" Uhr"</f>
         <v/>
       </c>
     </row>
     <row r="22" ht="20" customHeight="1">
-      <c r="B22" s="45" t="inlineStr">
+      <c r="B22" s="47" t="inlineStr">
         <is>
           <t>Name der Lehrkraft:</t>
         </is>
       </c>
-      <c r="C22" s="44">
+      <c r="C22" s="46">
         <f>Teilnehmer!C4</f>
         <v/>
       </c>
     </row>
     <row r="24" ht="20" customHeight="1">
-      <c r="B24" s="45" t="inlineStr">
+      <c r="B24" s="47" t="inlineStr">
         <is>
           <t>Verantwortlicher Arzt:</t>
         </is>
       </c>
-      <c r="C24" s="44">
+      <c r="C24" s="46">
         <f>Teilnehmer!C7</f>
         <v/>
       </c>
     </row>
     <row r="26" ht="20" customHeight="1">
-      <c r="B26" s="45" t="inlineStr">
+      <c r="B26" s="47" t="inlineStr">
         <is>
           <t>Masken-Charge:</t>
         </is>
       </c>
-      <c r="C26" s="48">
+      <c r="C26" s="50">
         <f>Teilnehmer!C8</f>
         <v/>
       </c>
     </row>
     <row r="28" ht="22" customHeight="1">
-      <c r="B28" s="42" t="inlineStr">
+      <c r="B28" s="44" t="inlineStr">
         <is>
           <t>Anzahl der Teilnehmenden</t>
         </is>
       </c>
     </row>
     <row r="30" ht="20" customHeight="1">
-      <c r="B30" s="45" t="inlineStr">
+      <c r="B30" s="47" t="inlineStr">
         <is>
           <t>Gesamtanzahl der Teilnehmenden:</t>
         </is>
       </c>
-      <c r="E30" s="49">
+      <c r="E30" s="51">
         <f>Teilnehmer!C32</f>
         <v/>
       </c>
     </row>
     <row r="31" ht="14" customHeight="1">
-      <c r="B31" s="43" t="inlineStr">
+      <c r="B31" s="45" t="inlineStr">
         <is>
           <t>(entspricht der Anzahl der Teilnehmerdatenblätter)</t>
         </is>
       </c>
     </row>
     <row r="33" ht="20" customHeight="1">
-      <c r="B33" s="45" t="inlineStr">
+      <c r="B33" s="47" t="inlineStr">
         <is>
           <t>davon betriebliche Ersthelfende:</t>
         </is>
       </c>
-      <c r="E33" s="49">
+      <c r="E33" s="51">
         <f>Teilnehmer!E32</f>
         <v/>
       </c>
     </row>
     <row r="35" ht="22" customHeight="1">
-      <c r="B35" s="42" t="inlineStr">
+      <c r="B35" s="44" t="inlineStr">
         <is>
           <t>Anlagen</t>
         </is>
       </c>
     </row>
     <row r="36" ht="16" customHeight="1">
-      <c r="B36" s="46" t="inlineStr">
+      <c r="B36" s="48" t="inlineStr">
         <is>
           <t>Alle Teilnehmenden sind mit Namen, Vornamen, Geburtsdatum und Unterschrift zu erfassen. Für UVT-Teilnehmende sind zusätzlich der Name und die Anschrift des Arbeitgebers sowie der kostentragende UVT zu ergänzen. Dies kann durch einzelne Teilnehmerdatenblätter erfolgen.</t>
         </is>
@@ -6491,43 +7825,43 @@
     <row r="37" ht="16" customHeight="1"/>
     <row r="38" ht="16" customHeight="1"/>
     <row r="40" ht="16" customHeight="1">
-      <c r="B40" s="46" t="inlineStr">
+      <c r="B40" s="48" t="inlineStr">
         <is>
           <t>Die Dokumentation ist fünf Jahre aufzubewahren und auf Anforderung dem Unfallversicherungsträger vorzulegen.</t>
         </is>
       </c>
     </row>
     <row r="42" ht="18" customHeight="1">
-      <c r="B42" s="45" t="inlineStr">
+      <c r="B42" s="47" t="inlineStr">
         <is>
           <t>Für die Richtigkeit der Angaben:</t>
         </is>
       </c>
     </row>
     <row r="47" ht="18" customHeight="1">
-      <c r="B47" s="50">
+      <c r="B47" s="52">
         <f>"Rastatt, "&amp;TEXT(Teilnehmer!C3,"DD.MM.YYYY")</f>
         <v/>
       </c>
-      <c r="E47" s="50">
+      <c r="E47" s="52">
         <f>"Rastatt, "&amp;TEXT(Teilnehmer!C3,"DD.MM.YYYY")</f>
         <v/>
       </c>
     </row>
     <row r="48" ht="14" customHeight="1">
-      <c r="B48" s="43" t="inlineStr">
+      <c r="B48" s="45" t="inlineStr">
         <is>
           <t>Ort, Datum     Unterschrift Lehrgangsleitung</t>
         </is>
       </c>
-      <c r="E48" s="43" t="inlineStr">
+      <c r="E48" s="45" t="inlineStr">
         <is>
           <t>Ort, Datum     Unterschrift Ausbildungsstelle</t>
         </is>
       </c>
     </row>
     <row r="50" ht="14" customHeight="1">
-      <c r="B50" s="51" t="inlineStr">
+      <c r="B50" s="53" t="inlineStr">
         <is>
           <t>Stand: 2026</t>
         </is>
@@ -6577,49 +7911,49 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="52" t="inlineStr">
+      <c r="A2" s="54" t="inlineStr">
         <is>
           <t>Putschler, Walter</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="52" t="inlineStr">
+      <c r="A3" s="54" t="inlineStr">
         <is>
           <t>Kaya, Michelle</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="52" t="inlineStr">
+      <c r="A4" s="54" t="inlineStr">
         <is>
           <t>Krempl, Elke</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="52" t="inlineStr">
+      <c r="A5" s="54" t="inlineStr">
         <is>
           <t>Breig, Bernd</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="52" t="inlineStr">
+      <c r="A6" s="54" t="inlineStr">
         <is>
           <t>Zuber, Harry</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="52" t="inlineStr">
+      <c r="A7" s="54" t="inlineStr">
         <is>
           <t>Jochim, Benjamin</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="52" t="inlineStr">
+      <c r="A8" s="54" t="inlineStr">
         <is>
           <t>Siebert, Emanuel</t>
         </is>

</xml_diff>

<commit_message>
Fix BG-Liste (one sheet) and Bescheinigungen (A4 landscape)
- BG-Liste: Combined Blatt1+Blatt2 into single sheet with page break
  at row 43, all 54 images with offset TwoCellAnchors for page 2
- Bescheinigungen: Changed from A3 to A4 landscape (2 certs per page)
- Removed BG-Liste_2 tab

https://claude.ai/code/session_0143BHkUCZBxvBT1DPHnv3wk
</commit_message>
<xml_diff>
--- a/EH_Kurs_2026.xlsx
+++ b/EH_Kurs_2026.xlsx
@@ -10,15 +10,12 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Teilnehmer" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bescheinigungen" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BG-Liste" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BG-Liste_2" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lehrgangsdoku" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hilfslisten" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lehrgangsdoku" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hilfslisten" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="Lehrkraefte">Hilfslisten!$A$2:$A$20</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'Bescheinigungen'!$A$1:$AZ$37</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="2">'BG-Liste'!$A$1:$E$51</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="3">'BG-Liste_2'!$A$1:$E$51</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="2">'BG-Liste'!$A$1:$E$86</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -3343,1114 +3340,812 @@
     </pic>
     <clientData/>
   </twoCellAnchor>
-</wsDr>
-</file>
-
-<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <twoCellAnchor editAs="oneCell">
+  <twoCellAnchor>
     <from>
       <col>0</col>
       <colOff>219075</colOff>
-      <row>7</row>
+      <row>50</row>
       <rowOff>0</rowOff>
     </from>
     <to>
       <col>1</col>
       <colOff>38174</colOff>
-      <row>19</row>
+      <row>62</row>
       <rowOff>29419</rowOff>
     </to>
     <pic>
       <nvPicPr>
-        <cNvPr id="2" name="Grafik 1"/>
-        <cNvPicPr>
-          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
-        </cNvPicPr>
+        <cNvPr id="28" name="Image 28" descr="Picture"/>
+        <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId28"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:off x="219075" y="3495675"/>
-          <a:ext cx="533474" cy="6049219"/>
-        </a:xfrm>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
-          <avLst/>
-        </a:prstGeom>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
   </twoCellAnchor>
-  <twoCellAnchor editAs="oneCell">
+  <twoCellAnchor>
     <from>
       <col>3</col>
       <colOff>2686050</colOff>
-      <row>8</row>
+      <row>51</row>
       <rowOff>409575</rowOff>
     </from>
     <to>
       <col>4</col>
       <colOff>1381322</colOff>
-      <row>19</row>
+      <row>62</row>
       <rowOff>210289</rowOff>
     </to>
     <pic>
       <nvPicPr>
-        <cNvPr id="3" name="Grafik 2"/>
-        <cNvPicPr>
-          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
-        </cNvPicPr>
+        <cNvPr id="29" name="Image 29" descr="Picture"/>
+        <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId29"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:off x="10134600" y="4429125"/>
-          <a:ext cx="1409897" cy="5296639"/>
-        </a:xfrm>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
-          <avLst/>
-        </a:prstGeom>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
   </twoCellAnchor>
-  <twoCellAnchor editAs="oneCell">
+  <twoCellAnchor>
     <from>
       <col>0</col>
       <colOff>190500</colOff>
-      <row>0</row>
+      <row>43</row>
       <rowOff>0</rowOff>
     </from>
     <to>
       <col>4</col>
       <colOff>1401762</colOff>
-      <row>4</row>
+      <row>47</row>
       <rowOff>19336</rowOff>
     </to>
     <pic>
       <nvPicPr>
-        <cNvPr id="4" name="Grafik 3"/>
-        <cNvPicPr>
-          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
-        </cNvPicPr>
+        <cNvPr id="30" name="Image 30" descr="Picture"/>
+        <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId30"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:off x="190500" y="0"/>
-          <a:ext cx="11374437" cy="2048161"/>
-        </a:xfrm>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
-          <avLst/>
-        </a:prstGeom>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
   </twoCellAnchor>
-  <twoCellAnchor editAs="oneCell">
+  <twoCellAnchor>
     <from>
       <col>0</col>
       <colOff>228600</colOff>
-      <row>0</row>
+      <row>43</row>
       <rowOff>19050</rowOff>
     </from>
     <to>
       <col>1</col>
       <colOff>28647</colOff>
-      <row>8</row>
+      <row>51</row>
       <rowOff>276822</rowOff>
     </to>
     <pic>
       <nvPicPr>
-        <cNvPr id="5" name="Grafik 4"/>
-        <cNvPicPr>
-          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
-        </cNvPicPr>
+        <cNvPr id="31" name="Image 31" descr="Picture"/>
+        <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4"/>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId31"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:off x="228600" y="19050"/>
-          <a:ext cx="514422" cy="4277322"/>
-        </a:xfrm>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
-          <avLst/>
-        </a:prstGeom>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
   </twoCellAnchor>
-  <twoCellAnchor editAs="oneCell">
+  <twoCellAnchor>
     <from>
       <col>0</col>
       <colOff>219075</colOff>
-      <row>6</row>
+      <row>49</row>
       <rowOff>400050</rowOff>
     </from>
     <to>
       <col>4</col>
       <colOff>1392232</colOff>
-      <row>9</row>
+      <row>52</row>
       <rowOff>114452</rowOff>
     </to>
     <pic>
       <nvPicPr>
-        <cNvPr id="6" name="Grafik 5"/>
-        <cNvPicPr>
-          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
-        </cNvPicPr>
+        <cNvPr id="32" name="Image 32" descr="Picture"/>
+        <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId5"/>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId32"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:off x="219075" y="3486150"/>
-          <a:ext cx="11336332" cy="1086002"/>
-        </a:xfrm>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
-          <avLst/>
-        </a:prstGeom>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
   </twoCellAnchor>
-  <twoCellAnchor editAs="oneCell">
+  <twoCellAnchor>
     <from>
       <col>0</col>
       <colOff>542925</colOff>
-      <row>4</row>
+      <row>47</row>
       <rowOff>495300</rowOff>
     </from>
     <to>
       <col>2</col>
       <colOff>1267607</colOff>
-      <row>5</row>
+      <row>48</row>
       <rowOff>276269</rowOff>
     </to>
     <pic>
       <nvPicPr>
-        <cNvPr id="7" name="Grafik 6"/>
-        <cNvPicPr>
-          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
-        </cNvPicPr>
+        <cNvPr id="33" name="Image 33" descr="Picture"/>
+        <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId6"/>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId33"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:off x="542925" y="2524125"/>
-          <a:ext cx="5601482" cy="314369"/>
-        </a:xfrm>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
-          <avLst/>
-        </a:prstGeom>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
   </twoCellAnchor>
-  <twoCellAnchor editAs="oneCell">
+  <twoCellAnchor>
     <from>
       <col>1</col>
       <colOff>3914775</colOff>
-      <row>2</row>
+      <row>45</row>
       <rowOff>476250</rowOff>
     </from>
     <to>
       <col>2</col>
       <colOff>1562353</colOff>
-      <row>7</row>
+      <row>50</row>
       <rowOff>219379</rowOff>
     </to>
     <pic>
       <nvPicPr>
-        <cNvPr id="8" name="Grafik 7"/>
-        <cNvPicPr>
-          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
-        </cNvPicPr>
+        <cNvPr id="34" name="Image 34" descr="Picture"/>
+        <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId7"/>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId34"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:off x="4629150" y="1533525"/>
-          <a:ext cx="1810003" cy="2181529"/>
-        </a:xfrm>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
-          <avLst/>
-        </a:prstGeom>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
   </twoCellAnchor>
-  <twoCellAnchor editAs="oneCell">
+  <twoCellAnchor>
     <from>
       <col>0</col>
       <colOff>285750</colOff>
-      <row>5</row>
+      <row>48</row>
       <rowOff>466725</rowOff>
     </from>
     <to>
       <col>2</col>
       <colOff>810379</colOff>
-      <row>6</row>
+      <row>49</row>
       <rowOff>181008</rowOff>
     </to>
     <pic>
       <nvPicPr>
-        <cNvPr id="9" name="Grafik 8"/>
-        <cNvPicPr>
-          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
-        </cNvPicPr>
+        <cNvPr id="35" name="Image 35" descr="Picture"/>
+        <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId8"/>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId35"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:off x="285750" y="3028950"/>
-          <a:ext cx="5401429" cy="238158"/>
-        </a:xfrm>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
-          <avLst/>
-        </a:prstGeom>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
   </twoCellAnchor>
-  <twoCellAnchor editAs="oneCell">
+  <twoCellAnchor>
     <from>
       <col>4</col>
       <colOff>942975</colOff>
-      <row>2</row>
+      <row>45</row>
       <rowOff>161925</rowOff>
     </from>
     <to>
       <col>4</col>
       <colOff>1381186</colOff>
-      <row>7</row>
+      <row>50</row>
       <rowOff>209897</rowOff>
     </to>
     <pic>
       <nvPicPr>
-        <cNvPr id="10" name="Grafik 9"/>
-        <cNvPicPr>
-          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
-        </cNvPicPr>
+        <cNvPr id="36" name="Image 36" descr="Picture"/>
+        <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId9"/>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId36"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:off x="11106150" y="1219200"/>
-          <a:ext cx="438211" cy="2486372"/>
-        </a:xfrm>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
-          <avLst/>
-        </a:prstGeom>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
   </twoCellAnchor>
-  <twoCellAnchor editAs="oneCell">
+  <twoCellAnchor>
     <from>
       <col>2</col>
       <colOff>1019175</colOff>
-      <row>5</row>
+      <row>48</row>
       <rowOff>142875</rowOff>
     </from>
     <to>
       <col>4</col>
       <colOff>1277124</colOff>
-      <row>5</row>
+      <row>48</row>
       <rowOff>447718</rowOff>
     </to>
     <pic>
       <nvPicPr>
-        <cNvPr id="11" name="Grafik 10"/>
-        <cNvPicPr>
-          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
-        </cNvPicPr>
+        <cNvPr id="37" name="Image 37" descr="Picture"/>
+        <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId10"/>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId37"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:off x="5895975" y="2705100"/>
-          <a:ext cx="5544324" cy="304843"/>
-        </a:xfrm>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
-          <avLst/>
-        </a:prstGeom>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
   </twoCellAnchor>
-  <twoCellAnchor editAs="oneCell">
+  <twoCellAnchor>
     <from>
       <col>2</col>
       <colOff>1047750</colOff>
-      <row>3</row>
+      <row>46</row>
       <rowOff>209550</rowOff>
     </from>
     <to>
       <col>4</col>
       <colOff>1172330</colOff>
-      <row>4</row>
+      <row>47</row>
       <rowOff>200091</rowOff>
     </to>
     <pic>
       <nvPicPr>
-        <cNvPr id="12" name="Grafik 11"/>
-        <cNvPicPr>
-          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
-        </cNvPicPr>
+        <cNvPr id="38" name="Image 38" descr="Picture"/>
+        <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId11"/>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId38"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:off x="5924550" y="1752600"/>
-          <a:ext cx="5410955" cy="476316"/>
-        </a:xfrm>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
-          <avLst/>
-        </a:prstGeom>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
   </twoCellAnchor>
-  <twoCellAnchor editAs="oneCell">
+  <twoCellAnchor>
     <from>
       <col>0</col>
       <colOff>200025</colOff>
-      <row>19</row>
+      <row>62</row>
       <rowOff>66675</rowOff>
     </from>
     <to>
       <col>4</col>
       <colOff>1392235</colOff>
-      <row>20</row>
+      <row>63</row>
       <rowOff>304908</rowOff>
     </to>
     <pic>
       <nvPicPr>
-        <cNvPr id="13" name="Grafik 12"/>
-        <cNvPicPr>
-          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
-        </cNvPicPr>
+        <cNvPr id="39" name="Image 39" descr="Picture"/>
+        <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId12"/>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId39"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:off x="200025" y="9582150"/>
-          <a:ext cx="11355385" cy="771633"/>
-        </a:xfrm>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
-          <avLst/>
-        </a:prstGeom>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
   </twoCellAnchor>
-  <twoCellAnchor editAs="oneCell">
+  <twoCellAnchor>
     <from>
       <col>0</col>
       <colOff>190500</colOff>
-      <row>20</row>
+      <row>63</row>
       <rowOff>47625</rowOff>
     </from>
     <to>
       <col>1</col>
       <colOff>857443</colOff>
-      <row>27</row>
+      <row>70</row>
       <rowOff>95632</rowOff>
     </to>
     <pic>
       <nvPicPr>
-        <cNvPr id="14" name="Grafik 13"/>
-        <cNvPicPr>
-          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
-        </cNvPicPr>
+        <cNvPr id="40" name="Image 40" descr="Picture"/>
+        <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId13"/>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId40"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:off x="190500" y="10096500"/>
-          <a:ext cx="1381318" cy="2734057"/>
-        </a:xfrm>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
-          <avLst/>
-        </a:prstGeom>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
   </twoCellAnchor>
-  <twoCellAnchor editAs="oneCell">
+  <twoCellAnchor>
     <from>
       <col>0</col>
       <colOff>171450</colOff>
-      <row>23</row>
+      <row>66</row>
       <rowOff>342900</rowOff>
     </from>
     <to>
       <col>2</col>
       <colOff>2058344</colOff>
-      <row>25</row>
+      <row>68</row>
       <rowOff>219168</rowOff>
     </to>
     <pic>
       <nvPicPr>
-        <cNvPr id="15" name="Grafik 14"/>
-        <cNvPicPr>
-          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
-        </cNvPicPr>
+        <cNvPr id="41" name="Image 41" descr="Picture"/>
+        <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId14"/>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId41"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:off x="171450" y="11563350"/>
-          <a:ext cx="6763694" cy="666843"/>
-        </a:xfrm>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
-          <avLst/>
-        </a:prstGeom>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
   </twoCellAnchor>
-  <twoCellAnchor editAs="oneCell">
+  <twoCellAnchor>
     <from>
       <col>2</col>
       <colOff>876300</colOff>
-      <row>20</row>
+      <row>63</row>
       <rowOff>38100</rowOff>
     </from>
     <to>
       <col>2</col>
       <colOff>1076353</colOff>
-      <row>25</row>
+      <row>68</row>
       <rowOff>19321</rowOff>
     </to>
     <pic>
       <nvPicPr>
-        <cNvPr id="16" name="Grafik 15"/>
-        <cNvPicPr>
-          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
-        </cNvPicPr>
+        <cNvPr id="42" name="Image 42" descr="Picture"/>
+        <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId15"/>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId42"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:off x="5753100" y="10086975"/>
-          <a:ext cx="200053" cy="1943371"/>
-        </a:xfrm>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
-          <avLst/>
-        </a:prstGeom>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
   </twoCellAnchor>
-  <twoCellAnchor editAs="oneCell">
+  <twoCellAnchor>
     <from>
       <col>2</col>
       <colOff>2057400</colOff>
-      <row>24</row>
+      <row>67</row>
       <rowOff>95250</rowOff>
     </from>
     <to>
       <col>3</col>
       <colOff>276335</colOff>
-      <row>25</row>
+      <row>68</row>
       <rowOff>28619</rowOff>
     </to>
     <pic>
       <nvPicPr>
-        <cNvPr id="17" name="Grafik 16"/>
-        <cNvPicPr>
-          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
-        </cNvPicPr>
+        <cNvPr id="43" name="Image 43" descr="Picture"/>
+        <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId16"/>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId43"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:off x="6934200" y="11725275"/>
-          <a:ext cx="790685" cy="314369"/>
-        </a:xfrm>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
-          <avLst/>
-        </a:prstGeom>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
   </twoCellAnchor>
-  <twoCellAnchor editAs="oneCell">
+  <twoCellAnchor>
     <from>
       <col>3</col>
       <colOff>209550</colOff>
-      <row>24</row>
+      <row>67</row>
       <rowOff>314325</rowOff>
     </from>
     <to>
       <col>4</col>
       <colOff>1372141</colOff>
-      <row>27</row>
+      <row>70</row>
       <rowOff>85847</rowOff>
     </to>
     <pic>
       <nvPicPr>
-        <cNvPr id="18" name="Grafik 17"/>
-        <cNvPicPr>
-          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
-        </cNvPicPr>
+        <cNvPr id="44" name="Image 44" descr="Picture"/>
+        <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId17"/>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId44"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:off x="7658100" y="11944350"/>
-          <a:ext cx="3877216" cy="876422"/>
-        </a:xfrm>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
-          <avLst/>
-        </a:prstGeom>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
   </twoCellAnchor>
-  <twoCellAnchor editAs="oneCell">
+  <twoCellAnchor>
     <from>
       <col>4</col>
       <colOff>904875</colOff>
-      <row>20</row>
+      <row>63</row>
       <rowOff>0</rowOff>
     </from>
     <to>
       <col>4</col>
       <colOff>1409770</colOff>
-      <row>25</row>
+      <row>68</row>
       <rowOff>200327</rowOff>
     </to>
     <pic>
       <nvPicPr>
-        <cNvPr id="19" name="Grafik 18"/>
-        <cNvPicPr>
-          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
-        </cNvPicPr>
+        <cNvPr id="45" name="Image 45" descr="Picture"/>
+        <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId18"/>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId45"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:off x="11068050" y="10048875"/>
-          <a:ext cx="504895" cy="2162477"/>
-        </a:xfrm>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
-          <avLst/>
-        </a:prstGeom>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
   </twoCellAnchor>
-  <twoCellAnchor editAs="oneCell">
+  <twoCellAnchor>
     <from>
       <col>0</col>
       <colOff>285750</colOff>
-      <row>25</row>
+      <row>68</row>
       <rowOff>60846</rowOff>
     </from>
     <to>
       <col>4</col>
       <colOff>1401749</colOff>
-      <row>27</row>
+      <row>70</row>
       <rowOff>97346</rowOff>
     </to>
     <pic>
       <nvPicPr>
-        <cNvPr id="20" name="Grafik 19"/>
-        <cNvPicPr>
-          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
-        </cNvPicPr>
+        <cNvPr id="46" name="Image 46" descr="Picture"/>
+        <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId19"/>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId46"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:off x="285750" y="12071871"/>
-          <a:ext cx="11279174" cy="760400"/>
-        </a:xfrm>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
-          <avLst/>
-        </a:prstGeom>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
   </twoCellAnchor>
-  <twoCellAnchor editAs="oneCell">
+  <twoCellAnchor>
     <from>
       <col>3</col>
       <colOff>2679539</colOff>
-      <row>25</row>
+      <row>68</row>
       <rowOff>265132</rowOff>
     </from>
     <to>
       <col>5</col>
       <colOff>3217</colOff>
-      <row>42</row>
+      <row>85</row>
       <rowOff>94584</rowOff>
     </to>
     <pic>
       <nvPicPr>
-        <cNvPr id="21" name="Grafik 20"/>
-        <cNvPicPr>
-          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
-        </cNvPicPr>
+        <cNvPr id="47" name="Image 47" descr="Picture"/>
+        <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId20"/>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId47"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:off x="10128089" y="12276157"/>
-          <a:ext cx="1457528" cy="4734827"/>
-        </a:xfrm>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
-          <avLst/>
-        </a:prstGeom>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
   </twoCellAnchor>
-  <twoCellAnchor editAs="oneCell">
+  <twoCellAnchor>
     <from>
       <col>0</col>
       <colOff>284664</colOff>
-      <row>31</row>
+      <row>74</row>
       <rowOff>54852</rowOff>
     </from>
     <to>
       <col>4</col>
       <colOff>590925</colOff>
-      <row>32</row>
+      <row>75</row>
       <rowOff>45363</rowOff>
     </to>
     <pic>
       <nvPicPr>
-        <cNvPr id="22" name="Grafik 21"/>
-        <cNvPicPr>
-          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
-        </cNvPicPr>
+        <cNvPr id="48" name="Image 48" descr="Picture"/>
+        <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId21"/>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId48"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:off x="284664" y="13751802"/>
-          <a:ext cx="10469436" cy="257211"/>
-        </a:xfrm>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
-          <avLst/>
-        </a:prstGeom>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
   </twoCellAnchor>
-  <twoCellAnchor editAs="oneCell">
+  <twoCellAnchor>
     <from>
       <col>2</col>
       <colOff>841214</colOff>
-      <row>27</row>
+      <row>70</row>
       <rowOff>43899</rowOff>
     </from>
     <to>
       <col>2</col>
       <colOff>993635</colOff>
-      <row>42</row>
+      <row>85</row>
       <rowOff>111408</rowOff>
     </to>
     <pic>
       <nvPicPr>
-        <cNvPr id="23" name="Grafik 22"/>
-        <cNvPicPr>
-          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
-        </cNvPicPr>
+        <cNvPr id="49" name="Image 49" descr="Picture"/>
+        <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId22"/>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId49"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:off x="5718014" y="12778824"/>
-          <a:ext cx="152421" cy="4248984"/>
-        </a:xfrm>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
-          <avLst/>
-        </a:prstGeom>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
   </twoCellAnchor>
-  <twoCellAnchor editAs="oneCell">
+  <twoCellAnchor>
     <from>
       <col>0</col>
       <colOff>192234</colOff>
-      <row>29</row>
+      <row>72</row>
       <rowOff>7900</rowOff>
     </from>
     <to>
       <col>4</col>
       <colOff>946233</colOff>
-      <row>30</row>
+      <row>73</row>
       <rowOff>55561</rowOff>
     </to>
     <pic>
       <nvPicPr>
-        <cNvPr id="24" name="Grafik 23"/>
-        <cNvPicPr>
-          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
-        </cNvPicPr>
+        <cNvPr id="50" name="Image 50" descr="Picture"/>
+        <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId23"/>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId50"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:off x="192234" y="13171450"/>
-          <a:ext cx="10917174" cy="257211"/>
-        </a:xfrm>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
-          <avLst/>
-        </a:prstGeom>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
   </twoCellAnchor>
-  <twoCellAnchor editAs="oneCell">
+  <twoCellAnchor>
     <from>
       <col>0</col>
       <colOff>180975</colOff>
-      <row>33</row>
+      <row>76</row>
       <rowOff>14208</rowOff>
     </from>
     <to>
       <col>4</col>
       <colOff>830184</colOff>
-      <row>34</row>
+      <row>77</row>
       <rowOff>99972</rowOff>
     </to>
     <pic>
       <nvPicPr>
-        <cNvPr id="25" name="Grafik 24"/>
-        <cNvPicPr>
-          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
-        </cNvPicPr>
+        <cNvPr id="51" name="Image 51" descr="Picture"/>
+        <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId24"/>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId51"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:off x="180975" y="14311233"/>
-          <a:ext cx="10812384" cy="276264"/>
-        </a:xfrm>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
-          <avLst/>
-        </a:prstGeom>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
   </twoCellAnchor>
-  <twoCellAnchor editAs="oneCell">
+  <twoCellAnchor>
     <from>
       <col>0</col>
       <colOff>193031</colOff>
-      <row>39</row>
+      <row>82</row>
       <rowOff>312275</rowOff>
     </from>
     <to>
       <col>4</col>
       <colOff>594555</colOff>
-      <row>42</row>
+      <row>85</row>
       <rowOff>112568</rowOff>
     </to>
     <pic>
       <nvPicPr>
-        <cNvPr id="26" name="Grafik 25"/>
-        <cNvPicPr>
-          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
-        </cNvPicPr>
+        <cNvPr id="52" name="Image 52" descr="Picture"/>
+        <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId25"/>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId52"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:off x="193031" y="16476200"/>
-          <a:ext cx="10564699" cy="552768"/>
-        </a:xfrm>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
-          <avLst/>
-        </a:prstGeom>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
   </twoCellAnchor>
-  <twoCellAnchor editAs="oneCell">
+  <twoCellAnchor>
     <from>
       <col>0</col>
       <colOff>171450</colOff>
-      <row>26</row>
+      <row>69</row>
       <rowOff>197975</rowOff>
     </from>
     <to>
       <col>0</col>
       <colOff>285766</colOff>
-      <row>40</row>
+      <row>83</row>
       <rowOff>198561</rowOff>
     </to>
     <pic>
       <nvPicPr>
-        <cNvPr id="27" name="Grafik 26"/>
-        <cNvPicPr>
-          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
-        </cNvPicPr>
+        <cNvPr id="53" name="Image 53" descr="Picture"/>
+        <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId26"/>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId53"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:off x="171450" y="12532850"/>
-          <a:ext cx="114316" cy="4201111"/>
-        </a:xfrm>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
-          <avLst/>
-        </a:prstGeom>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
   </twoCellAnchor>
-  <twoCellAnchor editAs="oneCell">
+  <twoCellAnchor>
     <from>
       <col>1</col>
       <colOff>304800</colOff>
-      <row>39</row>
+      <row>82</row>
       <rowOff>47625</rowOff>
     </from>
     <to>
       <col>1</col>
       <colOff>1028801</colOff>
-      <row>39</row>
+      <row>82</row>
       <rowOff>314362</rowOff>
     </to>
     <pic>
       <nvPicPr>
-        <cNvPr id="28" name="Grafik 27"/>
-        <cNvPicPr>
-          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
-        </cNvPicPr>
+        <cNvPr id="54" name="Image 54" descr="Picture"/>
+        <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId27"/>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId54"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:off x="1019175" y="16211550"/>
-          <a:ext cx="724001" cy="266737"/>
-        </a:xfrm>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
-          <avLst/>
-        </a:prstGeom>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -12208,7 +11903,7 @@
     <mergeCell ref="AV128:AZ128"/>
   </mergeCells>
   <pageMargins left="0.3149606299212598" right="0.3149606299212598" top="0.3937007874015748" bottom="0.3937007874015748" header="0.3149606299212598" footer="0.3149606299212598"/>
-  <pageSetup orientation="landscape" paperSize="8" fitToWidth="0"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToWidth="0"/>
   <rowBreaks count="8" manualBreakCount="8">
     <brk id="38" min="0" max="16383" man="1"/>
     <brk id="77" min="0" max="16383" man="1"/>
@@ -12230,7 +11925,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J40"/>
+  <dimension ref="A1:J83"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10.6640625" customWidth="1" min="1" max="1"/>
@@ -12541,359 +12236,335 @@
     <row r="41" ht="21" customHeight="1"/>
     <row r="42" ht="9" customHeight="1"/>
     <row r="43" ht="9" customHeight="1"/>
+    <row r="44" ht="42" customHeight="1"/>
+    <row r="45" ht="41.25" customHeight="1">
+      <c r="D45" s="35" t="n"/>
+      <c r="J45">
+        <f>IF(Teilnehmer!F3,Teilnehmer!F3,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46" ht="38.25" customHeight="1">
+      <c r="D46" s="35" t="n"/>
+    </row>
+    <row r="47" ht="38.25" customHeight="1">
+      <c r="D47" s="36" t="n"/>
+    </row>
+    <row r="48" ht="42" customHeight="1">
+      <c r="B48" s="37" t="inlineStr">
+        <is>
+          <t>Mercedes Benz AG</t>
+        </is>
+      </c>
+      <c r="D48" s="38" t="inlineStr">
+        <is>
+          <t>BG-Metall Nord-Süd</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="41.25" customHeight="1">
+      <c r="B49" s="39" t="inlineStr">
+        <is>
+          <t>Mercedsstr. 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="32.25" customHeight="1">
+      <c r="B50" s="39" t="inlineStr">
+        <is>
+          <t>76437 Rastatt</t>
+        </is>
+      </c>
+      <c r="D50" s="40" t="n">
+        <v>2.26255682176001e+19</v>
+      </c>
+    </row>
+    <row r="51" ht="41.25" customHeight="1">
+      <c r="D51" s="41" t="n"/>
+    </row>
+    <row r="52" ht="34.5" customHeight="1">
+      <c r="D52" s="36" t="n"/>
+    </row>
+    <row r="53" ht="39.75" customHeight="1">
+      <c r="A53" s="42" t="n">
+        <v>1</v>
+      </c>
+      <c r="B53" s="43">
+        <f>CONCATENATE(Teilnehmer!B21,", ",Teilnehmer!C21)</f>
+        <v/>
+      </c>
+      <c r="C53" s="44">
+        <f>IF(Teilnehmer!D21,Teilnehmer!D21,"")</f>
+        <v/>
+      </c>
+      <c r="D53" s="45" t="n"/>
+    </row>
+    <row r="54" ht="39.75" customHeight="1">
+      <c r="A54" s="42" t="n">
+        <v>2</v>
+      </c>
+      <c r="B54" s="43">
+        <f>CONCATENATE(Teilnehmer!B22,", ",Teilnehmer!C22)</f>
+        <v/>
+      </c>
+      <c r="C54" s="44">
+        <f>IF(Teilnehmer!D22,Teilnehmer!D22,"")</f>
+        <v/>
+      </c>
+      <c r="D54" s="46" t="n"/>
+    </row>
+    <row r="55" ht="39.75" customHeight="1">
+      <c r="A55" s="42" t="n">
+        <v>3</v>
+      </c>
+      <c r="B55" s="43">
+        <f>CONCATENATE(Teilnehmer!B23,", ",Teilnehmer!C23)</f>
+        <v/>
+      </c>
+      <c r="C55" s="44">
+        <f>IF(Teilnehmer!D23,Teilnehmer!D23,"")</f>
+        <v/>
+      </c>
+      <c r="D55" s="45" t="n"/>
+    </row>
+    <row r="56" ht="39.75" customHeight="1">
+      <c r="A56" s="42" t="n">
+        <v>4</v>
+      </c>
+      <c r="B56" s="43">
+        <f>CONCATENATE(Teilnehmer!B24,", ",Teilnehmer!C24)</f>
+        <v/>
+      </c>
+      <c r="C56" s="44">
+        <f>IF(Teilnehmer!D24,Teilnehmer!D24,"")</f>
+        <v/>
+      </c>
+      <c r="D56" s="45" t="n"/>
+    </row>
+    <row r="57" ht="40.5" customHeight="1">
+      <c r="A57" s="42" t="n">
+        <v>5</v>
+      </c>
+      <c r="B57" s="43">
+        <f>CONCATENATE(Teilnehmer!B25,", ",Teilnehmer!C25)</f>
+        <v/>
+      </c>
+      <c r="C57" s="44">
+        <f>IF(Teilnehmer!D25,Teilnehmer!D25,"")</f>
+        <v/>
+      </c>
+      <c r="D57" s="45" t="n"/>
+    </row>
+    <row r="58" ht="39.75" customHeight="1">
+      <c r="A58" s="42" t="n">
+        <v>6</v>
+      </c>
+      <c r="B58" s="43">
+        <f>CONCATENATE(Teilnehmer!B26,", ",Teilnehmer!C26)</f>
+        <v/>
+      </c>
+      <c r="C58" s="44">
+        <f>IF(Teilnehmer!D26,Teilnehmer!D26,"")</f>
+        <v/>
+      </c>
+      <c r="D58" s="45" t="n"/>
+    </row>
+    <row r="59" ht="40.5" customHeight="1">
+      <c r="A59" s="42" t="n">
+        <v>7</v>
+      </c>
+      <c r="B59" s="43">
+        <f>CONCATENATE(Teilnehmer!B27,", ",Teilnehmer!C27)</f>
+        <v/>
+      </c>
+      <c r="C59" s="44">
+        <f>IF(Teilnehmer!D27,Teilnehmer!D27,"")</f>
+        <v/>
+      </c>
+      <c r="D59" s="45" t="n"/>
+    </row>
+    <row r="60" ht="39" customHeight="1">
+      <c r="A60" s="42" t="n">
+        <v>8</v>
+      </c>
+      <c r="B60" s="43">
+        <f>CONCATENATE(Teilnehmer!B28,", ",Teilnehmer!C28)</f>
+        <v/>
+      </c>
+      <c r="C60" s="44">
+        <f>IF(Teilnehmer!D28,Teilnehmer!D28,"")</f>
+        <v/>
+      </c>
+      <c r="D60" s="45" t="n"/>
+    </row>
+    <row r="61" ht="39.75" customHeight="1">
+      <c r="A61" s="42" t="n">
+        <v>9</v>
+      </c>
+      <c r="B61" s="43">
+        <f>CONCATENATE(Teilnehmer!B29,", ",Teilnehmer!C29)</f>
+        <v/>
+      </c>
+      <c r="C61" s="44">
+        <f>IF(Teilnehmer!D29,Teilnehmer!D29,"")</f>
+        <v/>
+      </c>
+      <c r="D61" s="47" t="n"/>
+    </row>
+    <row r="62" ht="39.75" customHeight="1">
+      <c r="A62" s="42" t="n">
+        <v>10</v>
+      </c>
+      <c r="B62" s="43">
+        <f>CONCATENATE(Teilnehmer!B30,", ",Teilnehmer!C30)</f>
+        <v/>
+      </c>
+      <c r="C62" s="44">
+        <f>IF(Teilnehmer!D30,Teilnehmer!D30,"")</f>
+        <v/>
+      </c>
+      <c r="D62" s="45" t="n"/>
+    </row>
+    <row r="63" ht="42" customHeight="1"/>
+    <row r="64" ht="27.75" customHeight="1"/>
+    <row r="65" ht="32.25" customHeight="1">
+      <c r="B65" s="48" t="inlineStr">
+        <is>
+          <t>Dr. Schmidt, Sabine</t>
+        </is>
+      </c>
+    </row>
+    <row r="66" ht="32.25" customHeight="1">
+      <c r="B66" s="48" t="inlineStr">
+        <is>
+          <t>07222/91-22111</t>
+        </is>
+      </c>
+    </row>
+    <row r="67" ht="32.25" customHeight="1">
+      <c r="B67" s="55" t="inlineStr">
+        <is>
+          <t>sabine.m.schmidt@mercedes-benz.com</t>
+        </is>
+      </c>
+      <c r="D67" s="50" t="n"/>
+    </row>
+    <row r="68" ht="30" customHeight="1">
+      <c r="D68" s="51">
+        <f>Teilnehmer!C3</f>
+        <v/>
+      </c>
+    </row>
+    <row r="69" ht="25.5" customHeight="1"/>
+    <row r="70" ht="31.5" customHeight="1">
+      <c r="C70" s="51" t="n"/>
+    </row>
+    <row r="71" ht="8.25" customHeight="1"/>
+    <row r="72" ht="25.5" customHeight="1">
+      <c r="C72" s="51">
+        <f>Teilnehmer!C3</f>
+        <v/>
+      </c>
+    </row>
+    <row r="73" ht="16.5" customHeight="1"/>
+    <row r="74" ht="25.5" customHeight="1">
+      <c r="B74" s="52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  7.0103</t>
+        </is>
+      </c>
+      <c r="C74" s="50">
+        <f>Teilnehmer!C4</f>
+        <v/>
+      </c>
+    </row>
+    <row r="75" ht="21" customHeight="1">
+      <c r="B75" s="53" t="n"/>
+    </row>
+    <row r="76" ht="26.25" customHeight="1">
+      <c r="B76" s="54">
+        <f>"  "&amp;Teilnehmer!C5</f>
+        <v/>
+      </c>
+      <c r="C76" s="50" t="inlineStr">
+        <is>
+          <t>Mercedes Benz AG, PKW Werk</t>
+        </is>
+      </c>
+    </row>
+    <row r="77"/>
+    <row r="78"/>
+    <row r="79" ht="29.25" customHeight="1">
+      <c r="C79" s="50" t="inlineStr">
+        <is>
+          <t>Mercedes Benz AG</t>
+        </is>
+      </c>
+    </row>
+    <row r="80" ht="29.25" customHeight="1">
+      <c r="C80" s="50" t="inlineStr">
+        <is>
+          <t>Werksärztlicher Dienst</t>
+        </is>
+      </c>
+    </row>
+    <row r="81" ht="29.25" customHeight="1">
+      <c r="C81" s="50" t="inlineStr">
+        <is>
+          <t>PKW-Werk Rastatt</t>
+        </is>
+      </c>
+    </row>
+    <row r="82" ht="29.25" customHeight="1">
+      <c r="C82" s="50" t="inlineStr">
+        <is>
+          <t>Mercedesstraße 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="83" ht="29.25" customHeight="1">
+      <c r="B83" s="51">
+        <f>Teilnehmer!C3</f>
+        <v/>
+      </c>
+      <c r="C83" s="50" t="inlineStr">
+        <is>
+          <t>76437 Rastatt</t>
+        </is>
+      </c>
+    </row>
+    <row r="84" ht="21" customHeight="1"/>
+    <row r="85" ht="9" customHeight="1"/>
+    <row r="86" ht="9" customHeight="1"/>
   </sheetData>
-  <mergeCells count="8">
+  <mergeCells count="16">
+    <mergeCell ref="C83:D83"/>
     <mergeCell ref="C29:D29"/>
     <mergeCell ref="C38:D38"/>
+    <mergeCell ref="C80:D80"/>
+    <mergeCell ref="C72:D72"/>
+    <mergeCell ref="C82:D82"/>
     <mergeCell ref="C33:D33"/>
+    <mergeCell ref="C81:D81"/>
+    <mergeCell ref="C76:D76"/>
     <mergeCell ref="C37:D37"/>
     <mergeCell ref="C36:D36"/>
+    <mergeCell ref="C74:D74"/>
     <mergeCell ref="C40:D40"/>
     <mergeCell ref="C31:D31"/>
+    <mergeCell ref="C79:D79"/>
     <mergeCell ref="C39:D39"/>
   </mergeCells>
   <pageMargins left="0.1968503937007874" right="0.07874015748031496" top="0.3937007874015748" bottom="0.3937007874015748" header="0" footer="0"/>
   <pageSetup orientation="portrait" paperSize="9"/>
+  <rowBreaks count="1" manualBreakCount="1">
+    <brk id="43" min="0" max="16383" man="1"/>
+  </rowBreaks>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <tabColor rgb="00FF6F00"/>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:J40"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="10.6640625" customWidth="1" min="1" max="1"/>
-    <col width="62.44140625" customWidth="1" min="2" max="2"/>
-    <col width="38.5546875" customWidth="1" min="3" max="3"/>
-    <col width="40.6640625" customWidth="1" min="4" max="4"/>
-    <col width="21.33203125" customWidth="1" min="5" max="5"/>
-    <col width="4.33203125" customWidth="1" min="6" max="6"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="42" customHeight="1"/>
-    <row r="2" ht="41.25" customHeight="1">
-      <c r="D2" s="35" t="n"/>
-      <c r="J2">
-        <f>IF(Teilnehmer!F3,Teilnehmer!F3,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="3" ht="38.25" customHeight="1">
-      <c r="D3" s="35" t="n"/>
-    </row>
-    <row r="4" ht="38.25" customHeight="1">
-      <c r="D4" s="36" t="n"/>
-    </row>
-    <row r="5" ht="42" customHeight="1">
-      <c r="B5" s="37" t="inlineStr">
-        <is>
-          <t>Mercedes Benz AG</t>
-        </is>
-      </c>
-      <c r="D5" s="38" t="inlineStr">
-        <is>
-          <t>BG-Metall Nord-Süd</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="41.25" customHeight="1">
-      <c r="B6" s="39" t="inlineStr">
-        <is>
-          <t>Mercedsstr. 1</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="32.25" customHeight="1">
-      <c r="B7" s="39" t="inlineStr">
-        <is>
-          <t>76437 Rastatt</t>
-        </is>
-      </c>
-      <c r="D7" s="40" t="n">
-        <v>2.26255682176001e+19</v>
-      </c>
-    </row>
-    <row r="8" ht="41.25" customHeight="1">
-      <c r="D8" s="41" t="n"/>
-    </row>
-    <row r="9" ht="34.5" customHeight="1">
-      <c r="D9" s="36" t="n"/>
-    </row>
-    <row r="10" ht="39.75" customHeight="1">
-      <c r="A10" s="42" t="n">
-        <v>1</v>
-      </c>
-      <c r="B10" s="43">
-        <f>CONCATENATE(Teilnehmer!B21,", ",Teilnehmer!C21)</f>
-        <v/>
-      </c>
-      <c r="C10" s="44">
-        <f>IF(Teilnehmer!D21,Teilnehmer!D21,"")</f>
-        <v/>
-      </c>
-      <c r="D10" s="45" t="n"/>
-    </row>
-    <row r="11" ht="39.75" customHeight="1">
-      <c r="A11" s="42" t="n">
-        <v>2</v>
-      </c>
-      <c r="B11" s="43">
-        <f>CONCATENATE(Teilnehmer!B22,", ",Teilnehmer!C22)</f>
-        <v/>
-      </c>
-      <c r="C11" s="44">
-        <f>IF(Teilnehmer!D22,Teilnehmer!D22,"")</f>
-        <v/>
-      </c>
-      <c r="D11" s="46" t="n"/>
-    </row>
-    <row r="12" ht="39.75" customHeight="1">
-      <c r="A12" s="42" t="n">
-        <v>3</v>
-      </c>
-      <c r="B12" s="43">
-        <f>CONCATENATE(Teilnehmer!B23,", ",Teilnehmer!C23)</f>
-        <v/>
-      </c>
-      <c r="C12" s="44">
-        <f>IF(Teilnehmer!D23,Teilnehmer!D23,"")</f>
-        <v/>
-      </c>
-      <c r="D12" s="45" t="n"/>
-    </row>
-    <row r="13" ht="39.75" customHeight="1">
-      <c r="A13" s="42" t="n">
-        <v>4</v>
-      </c>
-      <c r="B13" s="43">
-        <f>CONCATENATE(Teilnehmer!B24,", ",Teilnehmer!C24)</f>
-        <v/>
-      </c>
-      <c r="C13" s="44">
-        <f>IF(Teilnehmer!D24,Teilnehmer!D24,"")</f>
-        <v/>
-      </c>
-      <c r="D13" s="45" t="n"/>
-    </row>
-    <row r="14" ht="40.5" customHeight="1">
-      <c r="A14" s="42" t="n">
-        <v>5</v>
-      </c>
-      <c r="B14" s="43">
-        <f>CONCATENATE(Teilnehmer!B25,", ",Teilnehmer!C25)</f>
-        <v/>
-      </c>
-      <c r="C14" s="44">
-        <f>IF(Teilnehmer!D25,Teilnehmer!D25,"")</f>
-        <v/>
-      </c>
-      <c r="D14" s="45" t="n"/>
-    </row>
-    <row r="15" ht="39.75" customHeight="1">
-      <c r="A15" s="42" t="n">
-        <v>6</v>
-      </c>
-      <c r="B15" s="43">
-        <f>CONCATENATE(Teilnehmer!B26,", ",Teilnehmer!C26)</f>
-        <v/>
-      </c>
-      <c r="C15" s="44">
-        <f>IF(Teilnehmer!D26,Teilnehmer!D26,"")</f>
-        <v/>
-      </c>
-      <c r="D15" s="45" t="n"/>
-    </row>
-    <row r="16" ht="40.5" customHeight="1">
-      <c r="A16" s="42" t="n">
-        <v>7</v>
-      </c>
-      <c r="B16" s="43">
-        <f>CONCATENATE(Teilnehmer!B27,", ",Teilnehmer!C27)</f>
-        <v/>
-      </c>
-      <c r="C16" s="44">
-        <f>IF(Teilnehmer!D27,Teilnehmer!D27,"")</f>
-        <v/>
-      </c>
-      <c r="D16" s="45" t="n"/>
-    </row>
-    <row r="17" ht="39" customHeight="1">
-      <c r="A17" s="42" t="n">
-        <v>8</v>
-      </c>
-      <c r="B17" s="43">
-        <f>CONCATENATE(Teilnehmer!B28,", ",Teilnehmer!C28)</f>
-        <v/>
-      </c>
-      <c r="C17" s="44">
-        <f>IF(Teilnehmer!D28,Teilnehmer!D28,"")</f>
-        <v/>
-      </c>
-      <c r="D17" s="45" t="n"/>
-    </row>
-    <row r="18" ht="39.75" customHeight="1">
-      <c r="A18" s="42" t="n">
-        <v>9</v>
-      </c>
-      <c r="B18" s="43">
-        <f>CONCATENATE(Teilnehmer!B29,", ",Teilnehmer!C29)</f>
-        <v/>
-      </c>
-      <c r="C18" s="44">
-        <f>IF(Teilnehmer!D29,Teilnehmer!D29,"")</f>
-        <v/>
-      </c>
-      <c r="D18" s="47" t="n"/>
-    </row>
-    <row r="19" ht="39.75" customHeight="1">
-      <c r="A19" s="42" t="n">
-        <v>10</v>
-      </c>
-      <c r="B19" s="43">
-        <f>CONCATENATE(Teilnehmer!B30,", ",Teilnehmer!C30)</f>
-        <v/>
-      </c>
-      <c r="C19" s="44">
-        <f>IF(Teilnehmer!D30,Teilnehmer!D30,"")</f>
-        <v/>
-      </c>
-      <c r="D19" s="45" t="n"/>
-    </row>
-    <row r="20" ht="42" customHeight="1"/>
-    <row r="21" ht="27.75" customHeight="1"/>
-    <row r="22" ht="32.25" customHeight="1">
-      <c r="B22" s="48" t="inlineStr">
-        <is>
-          <t>Dr. Schmidt, Sabine</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="32.25" customHeight="1">
-      <c r="B23" s="48" t="inlineStr">
-        <is>
-          <t>07222/91-22111</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="32.25" customHeight="1">
-      <c r="B24" s="55" t="inlineStr">
-        <is>
-          <t>sabine.m.schmidt@mercedes-benz.com</t>
-        </is>
-      </c>
-      <c r="D24" s="50" t="n"/>
-    </row>
-    <row r="25" ht="30" customHeight="1">
-      <c r="D25" s="51">
-        <f>Teilnehmer!C3</f>
-        <v/>
-      </c>
-    </row>
-    <row r="26" ht="25.5" customHeight="1"/>
-    <row r="27" ht="31.5" customHeight="1">
-      <c r="C27" s="51" t="n"/>
-    </row>
-    <row r="28" ht="8.25" customHeight="1"/>
-    <row r="29" ht="25.5" customHeight="1">
-      <c r="C29" s="51">
-        <f>Teilnehmer!C3</f>
-        <v/>
-      </c>
-    </row>
-    <row r="30" ht="16.5" customHeight="1"/>
-    <row r="31" ht="25.5" customHeight="1">
-      <c r="B31" s="52" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  7.0103</t>
-        </is>
-      </c>
-      <c r="C31" s="50">
-        <f>Teilnehmer!C4</f>
-        <v/>
-      </c>
-    </row>
-    <row r="32" ht="21" customHeight="1">
-      <c r="B32" s="53" t="n"/>
-    </row>
-    <row r="33" ht="26.25" customHeight="1">
-      <c r="B33" s="54">
-        <f>"  "&amp;Teilnehmer!C5</f>
-        <v/>
-      </c>
-      <c r="C33" s="50" t="inlineStr">
-        <is>
-          <t>Mercedes Benz AG, PKW Werk</t>
-        </is>
-      </c>
-    </row>
-    <row r="34"/>
-    <row r="35"/>
-    <row r="36" ht="29.25" customHeight="1">
-      <c r="C36" s="50" t="inlineStr">
-        <is>
-          <t>Mercedes Benz AG</t>
-        </is>
-      </c>
-    </row>
-    <row r="37" ht="29.25" customHeight="1">
-      <c r="C37" s="50" t="inlineStr">
-        <is>
-          <t>Werksärztlicher Dienst</t>
-        </is>
-      </c>
-    </row>
-    <row r="38" ht="29.25" customHeight="1">
-      <c r="C38" s="50" t="inlineStr">
-        <is>
-          <t>PKW-Werk Rastatt</t>
-        </is>
-      </c>
-    </row>
-    <row r="39" ht="29.25" customHeight="1">
-      <c r="C39" s="50" t="inlineStr">
-        <is>
-          <t>Mercedesstraße 1</t>
-        </is>
-      </c>
-    </row>
-    <row r="40" ht="29.25" customHeight="1">
-      <c r="B40" s="51">
-        <f>Teilnehmer!C3</f>
-        <v/>
-      </c>
-      <c r="C40" s="50" t="inlineStr">
-        <is>
-          <t>76437 Rastatt</t>
-        </is>
-      </c>
-    </row>
-    <row r="41" ht="21" customHeight="1"/>
-    <row r="42" ht="9" customHeight="1"/>
-    <row r="43" ht="9" customHeight="1"/>
-  </sheetData>
-  <mergeCells count="8">
-    <mergeCell ref="C29:D29"/>
-    <mergeCell ref="C38:D38"/>
-    <mergeCell ref="C33:D33"/>
-    <mergeCell ref="C37:D37"/>
-    <mergeCell ref="C36:D36"/>
-    <mergeCell ref="C40:D40"/>
-    <mergeCell ref="C31:D31"/>
-    <mergeCell ref="C39:D39"/>
-  </mergeCells>
-  <pageMargins left="0.1968503937007874" right="0.07874015748031496" top="0.3937007874015748" bottom="0.3937007874015748" header="0" footer="0"/>
-  <pageSetup orientation="portrait" paperSize="9"/>
-  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="006A1B9A"/>
@@ -13201,7 +12872,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="009E9E9E"/>

</xml_diff>

<commit_message>
Fix Bescheinigungen: set all 52 column widths explicitly
The original used XML column ranges (col min=1 max=25 width=2.71) which
openpyxl doesn't fully transfer. Now all 52 columns are set explicitly
to their original narrow widths so 2 certificates fit on A4 landscape.

https://claude.ai/code/session_0143BHkUCZBxvBT1DPHnv3wk
</commit_message>
<xml_diff>
--- a/EH_Kurs_2026.xlsx
+++ b/EH_Kurs_2026.xlsx
@@ -4826,9 +4826,57 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2.7109375" customWidth="1" min="1" max="1"/>
+    <col width="2.7109375" customWidth="1" min="2" max="2"/>
+    <col width="2.7109375" customWidth="1" min="3" max="3"/>
+    <col width="2.7109375" customWidth="1" min="4" max="4"/>
+    <col width="2.7109375" customWidth="1" min="5" max="5"/>
+    <col width="2.7109375" customWidth="1" min="6" max="6"/>
+    <col width="2.7109375" customWidth="1" min="7" max="7"/>
+    <col width="2.7109375" customWidth="1" min="8" max="8"/>
+    <col width="2.7109375" customWidth="1" min="9" max="9"/>
+    <col width="2.7109375" customWidth="1" min="10" max="10"/>
+    <col width="2.7109375" customWidth="1" min="11" max="11"/>
+    <col width="2.7109375" customWidth="1" min="12" max="12"/>
+    <col width="2.7109375" customWidth="1" min="13" max="13"/>
+    <col width="2.7109375" customWidth="1" min="14" max="14"/>
+    <col width="2.7109375" customWidth="1" min="15" max="15"/>
+    <col width="2.7109375" customWidth="1" min="16" max="16"/>
+    <col width="2.7109375" customWidth="1" min="17" max="17"/>
+    <col width="2.7109375" customWidth="1" min="18" max="18"/>
+    <col width="2.7109375" customWidth="1" min="19" max="19"/>
+    <col width="2.7109375" customWidth="1" min="20" max="20"/>
+    <col width="2.7109375" customWidth="1" min="21" max="21"/>
+    <col width="2.7109375" customWidth="1" min="22" max="22"/>
+    <col width="2.7109375" customWidth="1" min="23" max="23"/>
+    <col width="2.7109375" customWidth="1" min="24" max="24"/>
+    <col width="2.7109375" customWidth="1" min="25" max="25"/>
     <col width="2.42578125" customWidth="1" min="26" max="26"/>
+    <col width="2.42578125" customWidth="1" min="27" max="27"/>
     <col width="2.5703125" customWidth="1" min="28" max="28"/>
     <col width="2.7109375" customWidth="1" min="29" max="29"/>
+    <col width="2.7109375" customWidth="1" min="30" max="30"/>
+    <col width="2.7109375" customWidth="1" min="31" max="31"/>
+    <col width="2.7109375" customWidth="1" min="32" max="32"/>
+    <col width="2.7109375" customWidth="1" min="33" max="33"/>
+    <col width="2.7109375" customWidth="1" min="34" max="34"/>
+    <col width="2.7109375" customWidth="1" min="35" max="35"/>
+    <col width="2.7109375" customWidth="1" min="36" max="36"/>
+    <col width="2.7109375" customWidth="1" min="37" max="37"/>
+    <col width="2.7109375" customWidth="1" min="38" max="38"/>
+    <col width="2.7109375" customWidth="1" min="39" max="39"/>
+    <col width="2.7109375" customWidth="1" min="40" max="40"/>
+    <col width="2.7109375" customWidth="1" min="41" max="41"/>
+    <col width="2.7109375" customWidth="1" min="42" max="42"/>
+    <col width="2.7109375" customWidth="1" min="43" max="43"/>
+    <col width="2.7109375" customWidth="1" min="44" max="44"/>
+    <col width="2.7109375" customWidth="1" min="45" max="45"/>
+    <col width="2.7109375" customWidth="1" min="46" max="46"/>
+    <col width="2.7109375" customWidth="1" min="47" max="47"/>
+    <col width="2.7109375" customWidth="1" min="48" max="48"/>
+    <col width="2.7109375" customWidth="1" min="49" max="49"/>
+    <col width="2.7109375" customWidth="1" min="50" max="50"/>
+    <col width="2.7109375" customWidth="1" min="51" max="51"/>
+    <col width="2.7109375" customWidth="1" min="52" max="52"/>
     <col width="9.140625" customWidth="1" min="53" max="53"/>
     <col width="10.140625" customWidth="1" min="57" max="57"/>
     <col width="9.140625" customWidth="1" min="58" max="58"/>

</xml_diff>

<commit_message>
Fix Bescheinigungen print: fitToWidth=1 + fitToPage + print area
The certificates were showing "Keine Skalierung" (no scaling) causing
one certificate to fill the whole page. Now set fitToWidth=1 with
fitToPage=True so 52 narrow columns scale to fit A4 landscape, showing
2 certificates per page as in the original.

https://claude.ai/code/session_0143BHkUCZBxvBT1DPHnv3wk
</commit_message>
<xml_diff>
--- a/EH_Kurs_2026.xlsx
+++ b/EH_Kurs_2026.xlsx
@@ -15,6 +15,7 @@
   </sheets>
   <definedNames>
     <definedName name="Lehrkraefte">Hilfslisten!$A$2:$A$20</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'Bescheinigungen'!$A$1:$AZ$388</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="2">'BG-Liste'!$A$1:$E$86</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -4820,7 +4821,7 @@
   <sheetPr>
     <tabColor rgb="001B5E20"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:BE388"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -11951,7 +11952,7 @@
     <mergeCell ref="AV128:AZ128"/>
   </mergeCells>
   <pageMargins left="0.3149606299212598" right="0.3149606299212598" top="0.3937007874015748" bottom="0.3937007874015748" header="0.3149606299212598" footer="0.3149606299212598"/>
-  <pageSetup orientation="landscape" paperSize="9" fitToWidth="0"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
   <rowBreaks count="8" manualBreakCount="8">
     <brk id="38" min="0" max="16383" man="1"/>
     <brk id="77" min="0" max="16383" man="1"/>

</xml_diff>

<commit_message>
Fix Bescheinigungen blank pages: A3 paper, fitToPage, full print area
- Change paper size from A4 (9) to A3 (8) so certificates fit on one page
- Enable fitToWidth=1 + fitToPage so content scales to page width
- Expand print area from rows 1-37 to rows 1-388 (all 10 certificate pages)
- Add missing row break at 350 for proper page 9/10 separation
- Apply same fixes in post-processing to prevent XML overwrite

https://claude.ai/code/session_018GViNkkSVBF987eQMSRFgD
</commit_message>
<xml_diff>
--- a/EH_Kurs_2026.xlsx
+++ b/EH_Kurs_2026.xlsx
@@ -1,20 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Teilnehmer" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bescheinigungen" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BG-Liste" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lehrgangsdoku" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hilfslisten" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Teilnehmer" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Bescheinigungen" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="BG-Liste" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Lehrgangsdoku" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Hilfslisten" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="Lehrkraefte">Hilfslisten!$A$2:$A$20</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'Bescheinigungen'!$A$1:$AZ$37</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'Bescheinigungen'!$A$1:$AZ$388</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="2">'BG-Liste'!$A$1:$E$86</definedName>
   </definedNames>
   <calcPr calcId="191028" fullCalcOnLoad="1"/>
@@ -5713,7 +5713,7 @@
   <sheetPr>
     <tabColor rgb="001B5E20"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:BE388"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="14.25" customHeight="1"/>
@@ -12796,7 +12796,7 @@
     <mergeCell ref="AV128:AZ128"/>
   </mergeCells>
   <pageMargins left="0.31496062992125984" right="0.31496062992125984" top="0.39370078740157483" bottom="0.39370078740157483" header="0.31496062992125984" footer="0.31496062992125984"/>
-  <pageSetup paperSize="9" fitToWidth="0" orientation="landscape"/>
+  <pageSetup paperSize="8" fitToWidth="1" fitToHeight="0" orientation="landscape"/>
   <headerFooter>
     <oddHeader>&amp;L&amp;"CorpoS"&amp;1 &amp;K000000Internal#</oddHeader>
     <oddFooter/>
@@ -12805,7 +12805,7 @@
     <firstHeader/>
     <firstFooter/>
   </headerFooter>
-  <rowBreaks count="8" manualBreakCount="8">
+  <rowBreaks count="9" manualBreakCount="9">
     <brk id="38" min="0" max="16383" man="1"/>
     <brk id="77" min="0" max="16383" man="1"/>
     <brk id="116" min="0" max="16383" man="1"/>
@@ -12814,8 +12814,8 @@
     <brk id="233" min="0" max="16383" man="1"/>
     <brk id="272" min="0" max="16383" man="1"/>
     <brk id="311" min="0" max="16383" man="1"/>
+    <brk id="350" min="0" max="16383" man="1"/>
   </rowBreaks>
-  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -13461,7 +13461,6 @@
   <rowBreaks count="1" manualBreakCount="1">
     <brk id="43" min="0" max="16383" man="1"/>
   </rowBreaks>
-  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Fix Excel repair error: add drawing refs, sheet rels, and content types
The post-processing replaced drawings/images correctly but missed three
critical linkages that caused Excel to show a repair dialog on open:

- Add <drawing r:id="rId1"/> to Bescheinigungen and BG-Liste sheet XML
- Add xmlns:r namespace declaration to both worksheet root elements
- Create sheet2.xml.rels and sheet3.xml.rels linking sheets to drawings
- Add Content_Types entries for PNG images and drawing XML files

https://claude.ai/code/session_018GViNkkSVBF987eQMSRFgD
</commit_message>
<xml_diff>
--- a/EH_Kurs_2026.xlsx
+++ b/EH_Kurs_2026.xlsx
@@ -5709,7 +5709,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr>
     <tabColor rgb="001B5E20"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -12816,11 +12816,12 @@
     <brk id="311" min="0" max="16383" man="1"/>
     <brk id="350" min="0" max="16383" man="1"/>
   </rowBreaks>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr>
     <tabColor rgb="00FF6F00"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -13461,6 +13462,7 @@
   <rowBreaks count="1" manualBreakCount="1">
     <brk id="43" min="0" max="16383" man="1"/>
   </rowBreaks>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Fix page setup: A4 (not A3) for certs, add fitToPage for BG-Liste
- Revert Bescheinigungen from A3 back to A4 landscape with fitToWidth=1
  (2x A4 certificates side by side, slightly scaled to fit)
- Add fitToWidth=1 + fitToPage for BG-Liste (was missing, original had
  scale=56% with fitToPage - lost during copy_sheet)
- All sheets now have proper A4 page setup with fitToPage enabled

https://claude.ai/code/session_018GViNkkSVBF987eQMSRFgD
</commit_message>
<xml_diff>
--- a/EH_Kurs_2026.xlsx
+++ b/EH_Kurs_2026.xlsx
@@ -12796,7 +12796,7 @@
     <mergeCell ref="AV128:AZ128"/>
   </mergeCells>
   <pageMargins left="0.31496062992125984" right="0.31496062992125984" top="0.39370078740157483" bottom="0.39370078740157483" header="0.31496062992125984" footer="0.31496062992125984"/>
-  <pageSetup paperSize="8" fitToWidth="1" fitToHeight="0" orientation="landscape"/>
+  <pageSetup paperSize="9" fitToWidth="1" fitToHeight="0" orientation="landscape"/>
   <headerFooter>
     <oddHeader>&amp;L&amp;"CorpoS"&amp;1 &amp;K000000Internal#</oddHeader>
     <oddFooter/>
@@ -12825,7 +12825,7 @@
   <sheetPr>
     <tabColor rgb="00FF6F00"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:J83"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -13458,7 +13458,7 @@
     <mergeCell ref="C39:D39"/>
   </mergeCells>
   <pageMargins left="0.1968503937007874" right="0.07874015748031496" top="0.3937007874015748" bottom="0.3937007874015748" header="0" footer="0"/>
-  <pageSetup orientation="portrait" paperSize="9"/>
+  <pageSetup orientation="portrait" paperSize="9" fitToHeight="0" fitToWidth="1"/>
   <rowBreaks count="1" manualBreakCount="1">
     <brk id="43" min="0" max="16383" man="1"/>
   </rowBreaks>

</xml_diff>